<commit_message>
Trade logic changes, offers valued by net ratio instead of net value, complexity tier added to determine pick package size, added min_cost vs min_ratio roll to determine selected package to offer, fixed chained trade bug, future draft pick value tweaks
</commit_message>
<xml_diff>
--- a/Files/TestFiles/DraftPickValue.xlsx
+++ b/Files/TestFiles/DraftPickValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AC2BE56-21C9-4A94-A876-7F8B37135EFE}"/>
+  <xr:revisionPtr revIDLastSave="408" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80C7DC7F-6A88-4BEE-9773-2CE24AB368C8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B6B8C1A-1A59-46A0-9756-E6597FCDBA38}"/>
   </bookViews>
@@ -449,7 +449,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -471,7 +471,7 @@
         <v>3000</v>
       </c>
       <c r="C2" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -482,7 +482,7 @@
         <v>2600</v>
       </c>
       <c r="C3" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -493,7 +493,7 @@
         <v>2200</v>
       </c>
       <c r="C4" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -504,7 +504,7 @@
         <v>1800</v>
       </c>
       <c r="C5" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -515,7 +515,7 @@
         <v>1700</v>
       </c>
       <c r="C6" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -526,7 +526,7 @@
         <v>1600</v>
       </c>
       <c r="C7" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -537,7 +537,7 @@
         <v>1500</v>
       </c>
       <c r="C8" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -548,7 +548,7 @@
         <v>1400</v>
       </c>
       <c r="C9" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -559,7 +559,7 @@
         <v>1350</v>
       </c>
       <c r="C10" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -570,7 +570,7 @@
         <v>1300</v>
       </c>
       <c r="C11" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -581,7 +581,7 @@
         <v>1250</v>
       </c>
       <c r="C12" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -592,7 +592,7 @@
         <v>1200</v>
       </c>
       <c r="C13" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -603,7 +603,7 @@
         <v>1150</v>
       </c>
       <c r="C14" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -614,7 +614,7 @@
         <v>1100</v>
       </c>
       <c r="C15" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -625,7 +625,7 @@
         <v>1050</v>
       </c>
       <c r="C16" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -636,7 +636,7 @@
         <v>1000</v>
       </c>
       <c r="C17" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -647,7 +647,7 @@
         <v>950</v>
       </c>
       <c r="C18" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -658,7 +658,7 @@
         <v>900</v>
       </c>
       <c r="C19" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -669,7 +669,7 @@
         <v>875</v>
       </c>
       <c r="C20" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -680,7 +680,7 @@
         <v>850</v>
       </c>
       <c r="C21" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -691,7 +691,7 @@
         <v>800</v>
       </c>
       <c r="C22" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -702,7 +702,7 @@
         <v>780</v>
       </c>
       <c r="C23" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -713,7 +713,7 @@
         <v>760</v>
       </c>
       <c r="C24" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -724,7 +724,7 @@
         <v>740</v>
       </c>
       <c r="C25" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -735,7 +735,7 @@
         <v>720</v>
       </c>
       <c r="C26" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -746,7 +746,7 @@
         <v>700</v>
       </c>
       <c r="C27" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -757,7 +757,7 @@
         <v>680</v>
       </c>
       <c r="C28" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -768,7 +768,7 @@
         <v>660</v>
       </c>
       <c r="C29" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -779,7 +779,7 @@
         <v>640</v>
       </c>
       <c r="C30" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -790,7 +790,7 @@
         <v>620</v>
       </c>
       <c r="C31" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -801,7 +801,7 @@
         <v>600</v>
       </c>
       <c r="C32" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -812,7 +812,7 @@
         <v>590</v>
       </c>
       <c r="C33" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -823,7 +823,7 @@
         <v>580</v>
       </c>
       <c r="C34" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -834,7 +834,7 @@
         <v>560</v>
       </c>
       <c r="C35" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -845,7 +845,7 @@
         <v>550</v>
       </c>
       <c r="C36" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -856,7 +856,7 @@
         <v>540</v>
       </c>
       <c r="C37" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -867,7 +867,7 @@
         <v>530</v>
       </c>
       <c r="C38" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -878,7 +878,7 @@
         <v>520</v>
       </c>
       <c r="C39" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -889,7 +889,7 @@
         <v>510</v>
       </c>
       <c r="C40" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -900,7 +900,7 @@
         <v>500</v>
       </c>
       <c r="C41" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -911,7 +911,7 @@
         <v>490</v>
       </c>
       <c r="C42" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -922,7 +922,7 @@
         <v>480</v>
       </c>
       <c r="C43" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -933,7 +933,7 @@
         <v>470</v>
       </c>
       <c r="C44" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -944,7 +944,7 @@
         <v>460</v>
       </c>
       <c r="C45" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -955,7 +955,7 @@
         <v>450</v>
       </c>
       <c r="C46" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -966,7 +966,7 @@
         <v>440</v>
       </c>
       <c r="C47" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -977,7 +977,7 @@
         <v>430</v>
       </c>
       <c r="C48" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -988,7 +988,7 @@
         <v>420</v>
       </c>
       <c r="C49" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -999,7 +999,7 @@
         <v>410</v>
       </c>
       <c r="C50" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1010,7 +1010,7 @@
         <v>400</v>
       </c>
       <c r="C51" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1021,7 +1021,7 @@
         <v>390</v>
       </c>
       <c r="C52" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1032,7 +1032,7 @@
         <v>380</v>
       </c>
       <c r="C53" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1043,7 +1043,7 @@
         <v>370</v>
       </c>
       <c r="C54" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1054,7 +1054,7 @@
         <v>360</v>
       </c>
       <c r="C55" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1065,7 +1065,7 @@
         <v>350</v>
       </c>
       <c r="C56" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1076,7 +1076,7 @@
         <v>340</v>
       </c>
       <c r="C57" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1087,7 +1087,7 @@
         <v>330</v>
       </c>
       <c r="C58" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1098,7 +1098,7 @@
         <v>320</v>
       </c>
       <c r="C59" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1109,7 +1109,7 @@
         <v>310</v>
       </c>
       <c r="C60" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1120,7 +1120,7 @@
         <v>300</v>
       </c>
       <c r="C61" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1131,7 +1131,7 @@
         <v>292</v>
       </c>
       <c r="C62" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1142,7 +1142,7 @@
         <v>284</v>
       </c>
       <c r="C63" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1153,7 +1153,7 @@
         <v>276</v>
       </c>
       <c r="C64" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1164,7 +1164,7 @@
         <v>270</v>
       </c>
       <c r="C65" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,7 +1175,7 @@
         <v>265</v>
       </c>
       <c r="C66" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -1186,7 +1186,7 @@
         <v>260</v>
       </c>
       <c r="C67" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,7 +1197,7 @@
         <v>255</v>
       </c>
       <c r="C68" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1208,7 +1208,7 @@
         <v>250</v>
       </c>
       <c r="C69" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -1219,7 +1219,7 @@
         <v>245</v>
       </c>
       <c r="C70" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -1230,7 +1230,7 @@
         <v>240</v>
       </c>
       <c r="C71" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1241,7 +1241,7 @@
         <v>235</v>
       </c>
       <c r="C72" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1252,7 +1252,7 @@
         <v>230</v>
       </c>
       <c r="C73" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>225</v>
       </c>
       <c r="C74" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1274,7 +1274,7 @@
         <v>220</v>
       </c>
       <c r="C75" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>215</v>
       </c>
       <c r="C76" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1296,7 +1296,7 @@
         <v>210</v>
       </c>
       <c r="C77" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1307,7 +1307,7 @@
         <v>205</v>
       </c>
       <c r="C78" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1318,7 +1318,7 @@
         <v>200</v>
       </c>
       <c r="C79" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1329,7 +1329,7 @@
         <v>195</v>
       </c>
       <c r="C80" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1340,7 +1340,7 @@
         <v>190</v>
       </c>
       <c r="C81" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1351,7 +1351,7 @@
         <v>185</v>
       </c>
       <c r="C82" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1362,7 +1362,7 @@
         <v>180</v>
       </c>
       <c r="C83" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1373,7 +1373,7 @@
         <v>175</v>
       </c>
       <c r="C84" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1384,7 +1384,7 @@
         <v>170</v>
       </c>
       <c r="C85" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1395,7 +1395,7 @@
         <v>165</v>
       </c>
       <c r="C86" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1406,7 +1406,7 @@
         <v>160</v>
       </c>
       <c r="C87" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1417,7 +1417,7 @@
         <v>155</v>
       </c>
       <c r="C88" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1428,7 +1428,7 @@
         <v>150</v>
       </c>
       <c r="C89" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>145</v>
       </c>
       <c r="C90" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1450,7 +1450,7 @@
         <v>140</v>
       </c>
       <c r="C91" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -1461,7 +1461,7 @@
         <v>136</v>
       </c>
       <c r="C92" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -1472,7 +1472,7 @@
         <v>132</v>
       </c>
       <c r="C93" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -1483,7 +1483,7 @@
         <v>128</v>
       </c>
       <c r="C94" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -1494,7 +1494,7 @@
         <v>124</v>
       </c>
       <c r="C95" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -1505,7 +1505,7 @@
         <v>120</v>
       </c>
       <c r="C96" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -1516,7 +1516,7 @@
         <v>116</v>
       </c>
       <c r="C97" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>112</v>
       </c>
       <c r="C98" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -1538,7 +1538,7 @@
         <v>108</v>
       </c>
       <c r="C99" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>104</v>
       </c>
       <c r="C100" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -1560,7 +1560,7 @@
         <v>100</v>
       </c>
       <c r="C101" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -1571,7 +1571,7 @@
         <v>96</v>
       </c>
       <c r="C102" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -1582,7 +1582,7 @@
         <v>92</v>
       </c>
       <c r="C103" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -1593,7 +1593,7 @@
         <v>88</v>
       </c>
       <c r="C104" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -1604,7 +1604,7 @@
         <v>86</v>
       </c>
       <c r="C105" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>84</v>
       </c>
       <c r="C106" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -1626,7 +1626,7 @@
         <v>82</v>
       </c>
       <c r="C107" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -1637,7 +1637,7 @@
         <v>80</v>
       </c>
       <c r="C108" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -1648,7 +1648,7 @@
         <v>78</v>
       </c>
       <c r="C109" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -1659,7 +1659,7 @@
         <v>76</v>
       </c>
       <c r="C110" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -1670,7 +1670,7 @@
         <v>74</v>
       </c>
       <c r="C111" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -1681,7 +1681,7 @@
         <v>72</v>
       </c>
       <c r="C112" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -1692,7 +1692,7 @@
         <v>70</v>
       </c>
       <c r="C113" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
@@ -1703,7 +1703,7 @@
         <v>68</v>
       </c>
       <c r="C114" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -1714,7 +1714,7 @@
         <v>66</v>
       </c>
       <c r="C115" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -1725,7 +1725,7 @@
         <v>64</v>
       </c>
       <c r="C116" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
@@ -1736,7 +1736,7 @@
         <v>62</v>
       </c>
       <c r="C117" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -1747,7 +1747,7 @@
         <v>60</v>
       </c>
       <c r="C118" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -1758,7 +1758,7 @@
         <v>58</v>
       </c>
       <c r="C119" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -1769,7 +1769,7 @@
         <v>56</v>
       </c>
       <c r="C120" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -1780,7 +1780,7 @@
         <v>54</v>
       </c>
       <c r="C121" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -1791,7 +1791,7 @@
         <v>52</v>
       </c>
       <c r="C122" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -1802,7 +1802,7 @@
         <v>50</v>
       </c>
       <c r="C123" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -1813,7 +1813,7 @@
         <v>49</v>
       </c>
       <c r="C124" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -1824,7 +1824,7 @@
         <v>48</v>
       </c>
       <c r="C125" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -1835,7 +1835,7 @@
         <v>47</v>
       </c>
       <c r="C126" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -1846,7 +1846,7 @@
         <v>46</v>
       </c>
       <c r="C127" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
@@ -1857,7 +1857,7 @@
         <v>45</v>
       </c>
       <c r="C128" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -1868,7 +1868,7 @@
         <v>44</v>
       </c>
       <c r="C129" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -1879,7 +1879,7 @@
         <v>43</v>
       </c>
       <c r="C130" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
@@ -1890,7 +1890,7 @@
         <v>42</v>
       </c>
       <c r="C131" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -1901,7 +1901,7 @@
         <v>41</v>
       </c>
       <c r="C132" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -1912,7 +1912,7 @@
         <v>40</v>
       </c>
       <c r="C133" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -1923,7 +1923,7 @@
         <v>39</v>
       </c>
       <c r="C134" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -1934,7 +1934,7 @@
         <v>39</v>
       </c>
       <c r="C135" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -1945,7 +1945,7 @@
         <v>38</v>
       </c>
       <c r="C136" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -1956,7 +1956,7 @@
         <v>38</v>
       </c>
       <c r="C137" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -1967,7 +1967,7 @@
         <v>37</v>
       </c>
       <c r="C138" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -1978,7 +1978,7 @@
         <v>37</v>
       </c>
       <c r="C139" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -1989,7 +1989,7 @@
         <v>36</v>
       </c>
       <c r="C140" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -2000,7 +2000,7 @@
         <v>36</v>
       </c>
       <c r="C141" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
@@ -2011,7 +2011,7 @@
         <v>35</v>
       </c>
       <c r="C142" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -2022,7 +2022,7 @@
         <v>35</v>
       </c>
       <c r="C143" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -2033,7 +2033,7 @@
         <v>34</v>
       </c>
       <c r="C144" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
@@ -2044,7 +2044,7 @@
         <v>34</v>
       </c>
       <c r="C145" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -2055,7 +2055,7 @@
         <v>33</v>
       </c>
       <c r="C146" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -2066,7 +2066,7 @@
         <v>33</v>
       </c>
       <c r="C147" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -2077,7 +2077,7 @@
         <v>32</v>
       </c>
       <c r="C148" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
@@ -2088,7 +2088,7 @@
         <v>32</v>
       </c>
       <c r="C149" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -2099,7 +2099,7 @@
         <v>31</v>
       </c>
       <c r="C150" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -2110,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="C151" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -2121,7 +2121,7 @@
         <v>31</v>
       </c>
       <c r="C152" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -2132,7 +2132,7 @@
         <v>30</v>
       </c>
       <c r="C153" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -2143,7 +2143,7 @@
         <v>30</v>
       </c>
       <c r="C154" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
@@ -2154,7 +2154,7 @@
         <v>29</v>
       </c>
       <c r="C155" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
@@ -2165,7 +2165,7 @@
         <v>29</v>
       </c>
       <c r="C156" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -2176,7 +2176,7 @@
         <v>29</v>
       </c>
       <c r="C157" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -2187,7 +2187,7 @@
         <v>28</v>
       </c>
       <c r="C158" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
@@ -2198,7 +2198,7 @@
         <v>28</v>
       </c>
       <c r="C159" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
@@ -2209,7 +2209,7 @@
         <v>27</v>
       </c>
       <c r="C160" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -2220,7 +2220,7 @@
         <v>27</v>
       </c>
       <c r="C161" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -2231,7 +2231,7 @@
         <v>27</v>
       </c>
       <c r="C162" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
@@ -2242,7 +2242,7 @@
         <v>26</v>
       </c>
       <c r="C163" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -2253,7 +2253,7 @@
         <v>26</v>
       </c>
       <c r="C164" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -2264,7 +2264,7 @@
         <v>25</v>
       </c>
       <c r="C165" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -2275,7 +2275,7 @@
         <v>25</v>
       </c>
       <c r="C166" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -2286,7 +2286,7 @@
         <v>25</v>
       </c>
       <c r="C167" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -2297,7 +2297,7 @@
         <v>24</v>
       </c>
       <c r="C168" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -2308,7 +2308,7 @@
         <v>24</v>
       </c>
       <c r="C169" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -2319,7 +2319,7 @@
         <v>23</v>
       </c>
       <c r="C170" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -2330,7 +2330,7 @@
         <v>23</v>
       </c>
       <c r="C171" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -2341,7 +2341,7 @@
         <v>23</v>
       </c>
       <c r="C172" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -2352,7 +2352,7 @@
         <v>22</v>
       </c>
       <c r="C173" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -2363,7 +2363,7 @@
         <v>22</v>
       </c>
       <c r="C174" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -2374,7 +2374,7 @@
         <v>21</v>
       </c>
       <c r="C175" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -2385,7 +2385,7 @@
         <v>21</v>
       </c>
       <c r="C176" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -2396,7 +2396,7 @@
         <v>21</v>
       </c>
       <c r="C177" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -2407,7 +2407,7 @@
         <v>20</v>
       </c>
       <c r="C178" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -2418,7 +2418,7 @@
         <v>20</v>
       </c>
       <c r="C179" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -2429,7 +2429,7 @@
         <v>19</v>
       </c>
       <c r="C180" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -2440,7 +2440,7 @@
         <v>19</v>
       </c>
       <c r="C181" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -2451,7 +2451,7 @@
         <v>19</v>
       </c>
       <c r="C182" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -2462,7 +2462,7 @@
         <v>18</v>
       </c>
       <c r="C183" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -2473,7 +2473,7 @@
         <v>18</v>
       </c>
       <c r="C184" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -2484,7 +2484,7 @@
         <v>17</v>
       </c>
       <c r="C185" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -2495,7 +2495,7 @@
         <v>17</v>
       </c>
       <c r="C186" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
@@ -2506,7 +2506,7 @@
         <v>17</v>
       </c>
       <c r="C187" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -2517,7 +2517,7 @@
         <v>16</v>
       </c>
       <c r="C188" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -2528,7 +2528,7 @@
         <v>16</v>
       </c>
       <c r="C189" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -2539,7 +2539,7 @@
         <v>15</v>
       </c>
       <c r="C190" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -2550,7 +2550,7 @@
         <v>15</v>
       </c>
       <c r="C191" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -2561,7 +2561,7 @@
         <v>15</v>
       </c>
       <c r="C192" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -2572,7 +2572,7 @@
         <v>14</v>
       </c>
       <c r="C193" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
@@ -2583,7 +2583,7 @@
         <v>14</v>
       </c>
       <c r="C194" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -2594,7 +2594,7 @@
         <v>14</v>
       </c>
       <c r="C195" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -2605,7 +2605,7 @@
         <v>13</v>
       </c>
       <c r="C196" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -2616,7 +2616,7 @@
         <v>13</v>
       </c>
       <c r="C197" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -2627,7 +2627,7 @@
         <v>13</v>
       </c>
       <c r="C198" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -2638,7 +2638,7 @@
         <v>12</v>
       </c>
       <c r="C199" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -2649,7 +2649,7 @@
         <v>12</v>
       </c>
       <c r="C200" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -2660,7 +2660,7 @@
         <v>12</v>
       </c>
       <c r="C201" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
@@ -2671,7 +2671,7 @@
         <v>11</v>
       </c>
       <c r="C202" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -2682,7 +2682,7 @@
         <v>11</v>
       </c>
       <c r="C203" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -2693,7 +2693,7 @@
         <v>11</v>
       </c>
       <c r="C204" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -2704,7 +2704,7 @@
         <v>10</v>
       </c>
       <c r="C205" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -2715,7 +2715,7 @@
         <v>10</v>
       </c>
       <c r="C206" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -2726,7 +2726,7 @@
         <v>10</v>
       </c>
       <c r="C207" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -2737,7 +2737,7 @@
         <v>9</v>
       </c>
       <c r="C208" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
@@ -2748,7 +2748,7 @@
         <v>9</v>
       </c>
       <c r="C209" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
@@ -2803,7 +2803,7 @@
         <v>7</v>
       </c>
       <c r="C214" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -2814,7 +2814,7 @@
         <v>7</v>
       </c>
       <c r="C215" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -2825,7 +2825,7 @@
         <v>7</v>
       </c>
       <c r="C216" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -2836,7 +2836,7 @@
         <v>6</v>
       </c>
       <c r="C217" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
@@ -2847,7 +2847,7 @@
         <v>6</v>
       </c>
       <c r="C218" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
@@ -2858,7 +2858,7 @@
         <v>6</v>
       </c>
       <c r="C219" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
@@ -2869,7 +2869,7 @@
         <v>5</v>
       </c>
       <c r="C220" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -2880,7 +2880,7 @@
         <v>5</v>
       </c>
       <c r="C221" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
@@ -2891,7 +2891,7 @@
         <v>5</v>
       </c>
       <c r="C222" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
@@ -2902,7 +2902,7 @@
         <v>4</v>
       </c>
       <c r="C223" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
@@ -2913,7 +2913,7 @@
         <v>4</v>
       </c>
       <c r="C224" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -2924,7 +2924,7 @@
         <v>4</v>
       </c>
       <c r="C225" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
@@ -2935,7 +2935,7 @@
         <v>3</v>
       </c>
       <c r="C226" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
@@ -2946,7 +2946,7 @@
         <v>3</v>
       </c>
       <c r="C227" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
@@ -2957,7 +2957,7 @@
         <v>3</v>
       </c>
       <c r="C228" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
@@ -2968,7 +2968,7 @@
         <v>3</v>
       </c>
       <c r="C229" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
@@ -2979,7 +2979,7 @@
         <v>3</v>
       </c>
       <c r="C230" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
@@ -2990,7 +2990,7 @@
         <v>3</v>
       </c>
       <c r="C231" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
@@ -3001,7 +3001,7 @@
         <v>3</v>
       </c>
       <c r="C232" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
@@ -3012,7 +3012,7 @@
         <v>3</v>
       </c>
       <c r="C233" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -3023,7 +3023,7 @@
         <v>3</v>
       </c>
       <c r="C234" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
@@ -3034,7 +3034,7 @@
         <v>3</v>
       </c>
       <c r="C235" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
@@ -3350,7 +3350,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3358,7 +3358,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3366,7 +3366,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3374,7 +3374,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3382,7 +3382,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1">
-        <v>750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3390,7 +3390,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3398,7 +3398,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3406,7 +3406,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3414,7 +3414,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3422,7 +3422,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3430,7 +3430,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3438,7 +3438,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3446,7 +3446,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3454,7 +3454,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3462,7 +3462,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3470,7 +3470,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1">
-        <v>500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3478,7 +3478,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3486,7 +3486,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3494,7 +3494,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3502,7 +3502,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3510,7 +3510,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3518,7 +3518,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3526,7 +3526,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3534,7 +3534,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="1">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3542,7 +3542,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3550,7 +3550,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3558,7 +3558,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -3566,7 +3566,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3574,7 +3574,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3582,7 +3582,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -3590,7 +3590,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3598,7 +3598,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="1">
-        <v>350</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -3606,7 +3606,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -3614,7 +3614,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -3622,7 +3622,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3630,7 +3630,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -3638,7 +3638,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="1">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -3646,7 +3646,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -3654,7 +3654,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -3662,7 +3662,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3670,7 +3670,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3678,7 +3678,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="1">
-        <v>275</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -3686,7 +3686,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -3694,7 +3694,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -3702,7 +3702,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -3710,7 +3710,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -3718,7 +3718,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -3726,7 +3726,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="1">
-        <v>225</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -3734,7 +3734,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -3742,7 +3742,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -3750,7 +3750,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -3758,7 +3758,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="1">
-        <v>225</v>
+        <v>245</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -3766,7 +3766,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -3774,7 +3774,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -3782,7 +3782,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -3790,7 +3790,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="1">
-        <v>175</v>
+        <v>245</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -3798,7 +3798,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -3806,7 +3806,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -3814,7 +3814,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -3822,7 +3822,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -3838,7 +3838,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -3846,7 +3846,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -3854,7 +3854,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="1">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -3862,7 +3862,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -3870,7 +3870,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -3878,7 +3878,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -3886,7 +3886,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -3894,7 +3894,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="1">
-        <v>135</v>
+        <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -3902,7 +3902,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -3910,7 +3910,7 @@
         <v>70</v>
       </c>
       <c r="B72" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -3918,7 +3918,7 @@
         <v>71</v>
       </c>
       <c r="B73" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -3926,7 +3926,7 @@
         <v>72</v>
       </c>
       <c r="B74" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -3934,7 +3934,7 @@
         <v>73</v>
       </c>
       <c r="B75" s="1">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -3942,7 +3942,7 @@
         <v>74</v>
       </c>
       <c r="B76" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -3950,7 +3950,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -3958,7 +3958,7 @@
         <v>76</v>
       </c>
       <c r="B78" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -3966,7 +3966,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -3974,7 +3974,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -3982,7 +3982,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -3990,7 +3990,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -3998,7 +3998,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -4006,7 +4006,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -4014,7 +4014,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="1">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -4022,7 +4022,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -4030,7 +4030,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -4038,7 +4038,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -4046,7 +4046,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="1">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -4054,7 +4054,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -4062,7 +4062,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -4070,7 +4070,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -4078,7 +4078,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -4086,7 +4086,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -4094,7 +4094,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -4102,7 +4102,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -4110,7 +4110,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -4118,7 +4118,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -4126,7 +4126,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -4134,7 +4134,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -4142,7 +4142,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -4150,7 +4150,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -4158,7 +4158,7 @@
         <v>101</v>
       </c>
       <c r="B103" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -4166,7 +4166,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -4174,7 +4174,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -4182,7 +4182,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -4190,7 +4190,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
@@ -4198,7 +4198,7 @@
         <v>106</v>
       </c>
       <c r="B108" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
@@ -4206,7 +4206,7 @@
         <v>107</v>
       </c>
       <c r="B109" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -4214,7 +4214,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -4222,7 +4222,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -4230,7 +4230,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -4238,7 +4238,7 @@
         <v>111</v>
       </c>
       <c r="B113" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -4246,7 +4246,7 @@
         <v>112</v>
       </c>
       <c r="B114" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -4254,7 +4254,7 @@
         <v>113</v>
       </c>
       <c r="B115" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -4262,7 +4262,7 @@
         <v>114</v>
       </c>
       <c r="B116" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -4270,7 +4270,7 @@
         <v>115</v>
       </c>
       <c r="B117" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
@@ -4278,7 +4278,7 @@
         <v>116</v>
       </c>
       <c r="B118" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -4286,7 +4286,7 @@
         <v>117</v>
       </c>
       <c r="B119" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>118</v>
       </c>
       <c r="B120" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -4302,7 +4302,7 @@
         <v>119</v>
       </c>
       <c r="B121" s="1">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -4310,7 +4310,7 @@
         <v>120</v>
       </c>
       <c r="B122" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
@@ -4318,7 +4318,7 @@
         <v>121</v>
       </c>
       <c r="B123" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
@@ -4326,7 +4326,7 @@
         <v>122</v>
       </c>
       <c r="B124" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
@@ -4334,7 +4334,7 @@
         <v>123</v>
       </c>
       <c r="B125" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -4342,7 +4342,7 @@
         <v>124</v>
       </c>
       <c r="B126" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
@@ -4350,7 +4350,7 @@
         <v>125</v>
       </c>
       <c r="B127" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -4358,7 +4358,7 @@
         <v>126</v>
       </c>
       <c r="B128" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
@@ -4366,7 +4366,7 @@
         <v>127</v>
       </c>
       <c r="B129" s="1">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
@@ -4374,7 +4374,7 @@
         <v>128</v>
       </c>
       <c r="B130" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
@@ -4382,7 +4382,7 @@
         <v>129</v>
       </c>
       <c r="B131" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
@@ -4390,7 +4390,7 @@
         <v>130</v>
       </c>
       <c r="B132" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
@@ -4398,7 +4398,7 @@
         <v>131</v>
       </c>
       <c r="B133" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
@@ -4406,7 +4406,7 @@
         <v>132</v>
       </c>
       <c r="B134" s="1">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
@@ -4414,7 +4414,7 @@
         <v>133</v>
       </c>
       <c r="B135" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
@@ -4422,7 +4422,7 @@
         <v>134</v>
       </c>
       <c r="B136" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
@@ -4430,7 +4430,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -4438,7 +4438,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -4446,7 +4446,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="1">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
@@ -4454,7 +4454,7 @@
         <v>138</v>
       </c>
       <c r="B140" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -4462,7 +4462,7 @@
         <v>139</v>
       </c>
       <c r="B141" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -4470,7 +4470,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
@@ -4478,7 +4478,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
@@ -4486,7 +4486,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
@@ -4494,7 +4494,7 @@
         <v>143</v>
       </c>
       <c r="B145" s="1">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
@@ -4502,7 +4502,7 @@
         <v>144</v>
       </c>
       <c r="B146" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
@@ -4510,7 +4510,7 @@
         <v>145</v>
       </c>
       <c r="B147" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
@@ -4518,7 +4518,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -4534,7 +4534,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -4542,7 +4542,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -4550,7 +4550,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -4558,7 +4558,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -4566,7 +4566,7 @@
         <v>152</v>
       </c>
       <c r="B154" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -4574,7 +4574,7 @@
         <v>153</v>
       </c>
       <c r="B155" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -4582,7 +4582,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
@@ -4590,7 +4590,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
@@ -4598,7 +4598,7 @@
         <v>156</v>
       </c>
       <c r="B158" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -4606,7 +4606,7 @@
         <v>157</v>
       </c>
       <c r="B159" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
@@ -4614,7 +4614,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -4622,7 +4622,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
@@ -4630,7 +4630,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -4638,7 +4638,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -4646,7 +4646,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -4654,7 +4654,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
@@ -4662,7 +4662,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -4670,7 +4670,7 @@
         <v>165</v>
       </c>
       <c r="B167" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
@@ -4678,7 +4678,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -4686,7 +4686,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -4694,7 +4694,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
@@ -4702,7 +4702,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -4710,7 +4710,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -4718,7 +4718,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -4726,7 +4726,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -4734,7 +4734,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -4742,7 +4742,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -4750,7 +4750,7 @@
         <v>175</v>
       </c>
       <c r="B177" s="1">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
@@ -4766,7 +4766,7 @@
         <v>177</v>
       </c>
       <c r="B179" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -4774,7 +4774,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
@@ -4782,7 +4782,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
@@ -4790,7 +4790,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
@@ -4798,7 +4798,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
@@ -4806,7 +4806,7 @@
         <v>182</v>
       </c>
       <c r="B184" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
@@ -4814,7 +4814,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="1">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
@@ -4822,7 +4822,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -4830,7 +4830,7 @@
         <v>185</v>
       </c>
       <c r="B187" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
@@ -4838,7 +4838,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
@@ -4846,7 +4846,7 @@
         <v>187</v>
       </c>
       <c r="B189" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
@@ -4854,7 +4854,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
@@ -4862,7 +4862,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -4870,7 +4870,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
@@ -4878,7 +4878,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
@@ -4886,7 +4886,7 @@
         <v>192</v>
       </c>
       <c r="B194" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
@@ -4894,7 +4894,7 @@
         <v>193</v>
       </c>
       <c r="B195" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
@@ -4902,7 +4902,7 @@
         <v>194</v>
       </c>
       <c r="B196" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
@@ -4910,7 +4910,7 @@
         <v>195</v>
       </c>
       <c r="B197" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
@@ -4918,7 +4918,7 @@
         <v>196</v>
       </c>
       <c r="B198" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
@@ -4926,7 +4926,7 @@
         <v>197</v>
       </c>
       <c r="B199" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
@@ -4934,7 +4934,7 @@
         <v>198</v>
       </c>
       <c r="B200" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -4942,7 +4942,7 @@
         <v>199</v>
       </c>
       <c r="B201" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -4950,7 +4950,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
@@ -4958,7 +4958,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
@@ -4966,7 +4966,7 @@
         <v>202</v>
       </c>
       <c r="B204" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
@@ -4974,7 +4974,7 @@
         <v>203</v>
       </c>
       <c r="B205" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
@@ -4982,7 +4982,7 @@
         <v>204</v>
       </c>
       <c r="B206" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>205</v>
       </c>
       <c r="B207" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
@@ -4998,7 +4998,7 @@
         <v>206</v>
       </c>
       <c r="B208" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
@@ -5006,7 +5006,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
@@ -5046,7 +5046,7 @@
         <v>212</v>
       </c>
       <c r="B214" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
@@ -5054,7 +5054,7 @@
         <v>213</v>
       </c>
       <c r="B215" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
@@ -5062,7 +5062,7 @@
         <v>214</v>
       </c>
       <c r="B216" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
@@ -5070,7 +5070,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -5078,7 +5078,7 @@
         <v>216</v>
       </c>
       <c r="B218" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -5086,7 +5086,7 @@
         <v>217</v>
       </c>
       <c r="B219" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -5094,7 +5094,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -5102,7 +5102,7 @@
         <v>219</v>
       </c>
       <c r="B221" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -5110,7 +5110,7 @@
         <v>220</v>
       </c>
       <c r="B222" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -5118,7 +5118,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
@@ -5126,7 +5126,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
@@ -5134,7 +5134,7 @@
         <v>223</v>
       </c>
       <c r="B225" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
@@ -5142,7 +5142,7 @@
         <v>224</v>
       </c>
       <c r="B226" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
@@ -5150,7 +5150,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
@@ -5158,7 +5158,7 @@
         <v>226</v>
       </c>
       <c r="B228" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
@@ -5166,7 +5166,7 @@
         <v>227</v>
       </c>
       <c r="B229" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
@@ -5174,7 +5174,7 @@
         <v>228</v>
       </c>
       <c r="B230" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
@@ -5182,7 +5182,7 @@
         <v>229</v>
       </c>
       <c r="B231" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -5190,7 +5190,7 @@
         <v>230</v>
       </c>
       <c r="B232" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
@@ -5198,7 +5198,7 @@
         <v>231</v>
       </c>
       <c r="B233" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -5206,7 +5206,7 @@
         <v>232</v>
       </c>
       <c r="B234" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
@@ -5214,7 +5214,7 @@
         <v>233</v>
       </c>
       <c r="B235" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Tighten future-pick offer gates and R1 anchor rules, update future pick values
</commit_message>
<xml_diff>
--- a/Files/TestFiles/DraftPickValue.xlsx
+++ b/Files/TestFiles/DraftPickValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="408" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80C7DC7F-6A88-4BEE-9773-2CE24AB368C8}"/>
+  <xr:revisionPtr revIDLastSave="617" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF9FAFB-2AF4-4E17-A89D-BCA96B683724}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B6B8C1A-1A59-46A0-9756-E6597FCDBA38}"/>
   </bookViews>
@@ -933,7 +933,7 @@
         <v>470</v>
       </c>
       <c r="C44" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -944,7 +944,7 @@
         <v>460</v>
       </c>
       <c r="C45" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -955,7 +955,7 @@
         <v>450</v>
       </c>
       <c r="C46" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -966,7 +966,7 @@
         <v>440</v>
       </c>
       <c r="C47" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -977,7 +977,7 @@
         <v>430</v>
       </c>
       <c r="C48" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -988,7 +988,7 @@
         <v>420</v>
       </c>
       <c r="C49" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1087,7 +1087,7 @@
         <v>330</v>
       </c>
       <c r="C58" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1098,7 +1098,7 @@
         <v>320</v>
       </c>
       <c r="C59" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1109,7 +1109,7 @@
         <v>310</v>
       </c>
       <c r="C60" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1120,7 +1120,7 @@
         <v>300</v>
       </c>
       <c r="C61" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1131,7 +1131,7 @@
         <v>292</v>
       </c>
       <c r="C62" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1142,7 +1142,7 @@
         <v>284</v>
       </c>
       <c r="C63" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1153,7 +1153,7 @@
         <v>276</v>
       </c>
       <c r="C64" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1164,7 +1164,7 @@
         <v>270</v>
       </c>
       <c r="C65" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,7 +1175,7 @@
         <v>265</v>
       </c>
       <c r="C66" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -1186,7 +1186,7 @@
         <v>260</v>
       </c>
       <c r="C67" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,7 +1197,7 @@
         <v>255</v>
       </c>
       <c r="C68" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1208,7 +1208,7 @@
         <v>250</v>
       </c>
       <c r="C69" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -1219,7 +1219,7 @@
         <v>245</v>
       </c>
       <c r="C70" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -1230,7 +1230,7 @@
         <v>240</v>
       </c>
       <c r="C71" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1241,7 +1241,7 @@
         <v>235</v>
       </c>
       <c r="C72" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1252,7 +1252,7 @@
         <v>230</v>
       </c>
       <c r="C73" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>225</v>
       </c>
       <c r="C74" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1274,7 +1274,7 @@
         <v>220</v>
       </c>
       <c r="C75" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>215</v>
       </c>
       <c r="C76" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1296,7 +1296,7 @@
         <v>210</v>
       </c>
       <c r="C77" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1307,7 +1307,7 @@
         <v>205</v>
       </c>
       <c r="C78" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1318,7 +1318,7 @@
         <v>200</v>
       </c>
       <c r="C79" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1329,7 +1329,7 @@
         <v>195</v>
       </c>
       <c r="C80" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1340,7 +1340,7 @@
         <v>190</v>
       </c>
       <c r="C81" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1351,7 +1351,7 @@
         <v>185</v>
       </c>
       <c r="C82" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1362,7 +1362,7 @@
         <v>180</v>
       </c>
       <c r="C83" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1373,7 +1373,7 @@
         <v>175</v>
       </c>
       <c r="C84" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1384,7 +1384,7 @@
         <v>170</v>
       </c>
       <c r="C85" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1395,7 +1395,7 @@
         <v>165</v>
       </c>
       <c r="C86" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1406,7 +1406,7 @@
         <v>160</v>
       </c>
       <c r="C87" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1417,7 +1417,7 @@
         <v>155</v>
       </c>
       <c r="C88" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1428,7 +1428,7 @@
         <v>150</v>
       </c>
       <c r="C89" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>145</v>
       </c>
       <c r="C90" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1450,7 +1450,7 @@
         <v>140</v>
       </c>
       <c r="C91" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -1461,7 +1461,7 @@
         <v>136</v>
       </c>
       <c r="C92" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -1472,7 +1472,7 @@
         <v>132</v>
       </c>
       <c r="C93" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -1483,7 +1483,7 @@
         <v>128</v>
       </c>
       <c r="C94" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -1494,7 +1494,7 @@
         <v>124</v>
       </c>
       <c r="C95" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -1505,7 +1505,7 @@
         <v>120</v>
       </c>
       <c r="C96" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -1516,7 +1516,7 @@
         <v>116</v>
       </c>
       <c r="C97" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>112</v>
       </c>
       <c r="C98" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -1538,7 +1538,7 @@
         <v>108</v>
       </c>
       <c r="C99" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>104</v>
       </c>
       <c r="C100" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -1560,7 +1560,7 @@
         <v>100</v>
       </c>
       <c r="C101" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -1571,7 +1571,7 @@
         <v>96</v>
       </c>
       <c r="C102" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -1582,7 +1582,7 @@
         <v>92</v>
       </c>
       <c r="C103" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -1593,7 +1593,7 @@
         <v>88</v>
       </c>
       <c r="C104" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -1604,7 +1604,7 @@
         <v>86</v>
       </c>
       <c r="C105" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>84</v>
       </c>
       <c r="C106" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -1626,7 +1626,7 @@
         <v>82</v>
       </c>
       <c r="C107" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -1637,7 +1637,7 @@
         <v>80</v>
       </c>
       <c r="C108" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -1648,7 +1648,7 @@
         <v>78</v>
       </c>
       <c r="C109" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -1659,7 +1659,7 @@
         <v>76</v>
       </c>
       <c r="C110" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -1670,7 +1670,7 @@
         <v>74</v>
       </c>
       <c r="C111" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -1681,7 +1681,7 @@
         <v>72</v>
       </c>
       <c r="C112" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -1692,7 +1692,7 @@
         <v>70</v>
       </c>
       <c r="C113" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
@@ -1703,7 +1703,7 @@
         <v>68</v>
       </c>
       <c r="C114" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -1714,7 +1714,7 @@
         <v>66</v>
       </c>
       <c r="C115" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -1725,7 +1725,7 @@
         <v>64</v>
       </c>
       <c r="C116" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
@@ -1736,7 +1736,7 @@
         <v>62</v>
       </c>
       <c r="C117" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -1747,7 +1747,7 @@
         <v>60</v>
       </c>
       <c r="C118" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -1758,7 +1758,7 @@
         <v>58</v>
       </c>
       <c r="C119" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -1769,7 +1769,7 @@
         <v>56</v>
       </c>
       <c r="C120" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -1780,7 +1780,7 @@
         <v>54</v>
       </c>
       <c r="C121" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -1791,7 +1791,7 @@
         <v>52</v>
       </c>
       <c r="C122" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -1802,7 +1802,7 @@
         <v>50</v>
       </c>
       <c r="C123" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -1813,7 +1813,7 @@
         <v>49</v>
       </c>
       <c r="C124" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -1824,7 +1824,7 @@
         <v>48</v>
       </c>
       <c r="C125" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -1835,7 +1835,7 @@
         <v>47</v>
       </c>
       <c r="C126" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -1846,7 +1846,7 @@
         <v>46</v>
       </c>
       <c r="C127" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
@@ -1857,7 +1857,7 @@
         <v>45</v>
       </c>
       <c r="C128" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -1868,7 +1868,7 @@
         <v>44</v>
       </c>
       <c r="C129" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -1879,7 +1879,7 @@
         <v>43</v>
       </c>
       <c r="C130" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
@@ -1890,7 +1890,7 @@
         <v>42</v>
       </c>
       <c r="C131" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -1901,7 +1901,7 @@
         <v>41</v>
       </c>
       <c r="C132" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -1912,7 +1912,7 @@
         <v>40</v>
       </c>
       <c r="C133" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -1923,7 +1923,7 @@
         <v>39</v>
       </c>
       <c r="C134" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -1934,7 +1934,7 @@
         <v>39</v>
       </c>
       <c r="C135" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -1945,7 +1945,7 @@
         <v>38</v>
       </c>
       <c r="C136" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -1956,7 +1956,7 @@
         <v>38</v>
       </c>
       <c r="C137" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -1967,7 +1967,7 @@
         <v>37</v>
       </c>
       <c r="C138" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -1978,7 +1978,7 @@
         <v>37</v>
       </c>
       <c r="C139" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -1989,7 +1989,7 @@
         <v>36</v>
       </c>
       <c r="C140" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -2000,7 +2000,7 @@
         <v>36</v>
       </c>
       <c r="C141" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
@@ -2011,7 +2011,7 @@
         <v>35</v>
       </c>
       <c r="C142" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -2022,7 +2022,7 @@
         <v>35</v>
       </c>
       <c r="C143" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -2033,7 +2033,7 @@
         <v>34</v>
       </c>
       <c r="C144" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
@@ -2044,7 +2044,7 @@
         <v>34</v>
       </c>
       <c r="C145" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -2055,7 +2055,7 @@
         <v>33</v>
       </c>
       <c r="C146" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -2066,7 +2066,7 @@
         <v>33</v>
       </c>
       <c r="C147" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -2077,7 +2077,7 @@
         <v>32</v>
       </c>
       <c r="C148" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
@@ -2088,7 +2088,7 @@
         <v>32</v>
       </c>
       <c r="C149" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -2099,7 +2099,7 @@
         <v>31</v>
       </c>
       <c r="C150" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -2110,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="C151" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
@@ -2121,7 +2121,7 @@
         <v>31</v>
       </c>
       <c r="C152" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -2132,7 +2132,7 @@
         <v>30</v>
       </c>
       <c r="C153" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -2143,7 +2143,7 @@
         <v>30</v>
       </c>
       <c r="C154" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
@@ -2154,7 +2154,7 @@
         <v>29</v>
       </c>
       <c r="C155" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
@@ -2165,7 +2165,7 @@
         <v>29</v>
       </c>
       <c r="C156" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -2176,7 +2176,7 @@
         <v>29</v>
       </c>
       <c r="C157" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -2187,7 +2187,7 @@
         <v>28</v>
       </c>
       <c r="C158" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
@@ -2198,7 +2198,7 @@
         <v>28</v>
       </c>
       <c r="C159" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
@@ -2209,7 +2209,7 @@
         <v>27</v>
       </c>
       <c r="C160" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -2220,7 +2220,7 @@
         <v>27</v>
       </c>
       <c r="C161" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -2231,7 +2231,7 @@
         <v>27</v>
       </c>
       <c r="C162" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
@@ -2242,7 +2242,7 @@
         <v>26</v>
       </c>
       <c r="C163" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -2253,7 +2253,7 @@
         <v>26</v>
       </c>
       <c r="C164" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -2264,7 +2264,7 @@
         <v>25</v>
       </c>
       <c r="C165" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -2275,7 +2275,7 @@
         <v>25</v>
       </c>
       <c r="C166" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -2286,7 +2286,7 @@
         <v>25</v>
       </c>
       <c r="C167" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -2297,7 +2297,7 @@
         <v>24</v>
       </c>
       <c r="C168" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -2308,7 +2308,7 @@
         <v>24</v>
       </c>
       <c r="C169" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -2319,7 +2319,7 @@
         <v>23</v>
       </c>
       <c r="C170" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -2330,7 +2330,7 @@
         <v>23</v>
       </c>
       <c r="C171" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -2341,7 +2341,7 @@
         <v>23</v>
       </c>
       <c r="C172" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -2352,7 +2352,7 @@
         <v>22</v>
       </c>
       <c r="C173" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -2363,7 +2363,7 @@
         <v>22</v>
       </c>
       <c r="C174" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -2374,7 +2374,7 @@
         <v>21</v>
       </c>
       <c r="C175" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -2385,7 +2385,7 @@
         <v>21</v>
       </c>
       <c r="C176" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -2396,7 +2396,7 @@
         <v>21</v>
       </c>
       <c r="C177" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -2407,7 +2407,7 @@
         <v>20</v>
       </c>
       <c r="C178" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -2418,7 +2418,7 @@
         <v>20</v>
       </c>
       <c r="C179" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -2429,7 +2429,7 @@
         <v>19</v>
       </c>
       <c r="C180" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -2440,7 +2440,7 @@
         <v>19</v>
       </c>
       <c r="C181" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -2451,7 +2451,7 @@
         <v>19</v>
       </c>
       <c r="C182" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -2462,7 +2462,7 @@
         <v>18</v>
       </c>
       <c r="C183" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -2473,7 +2473,7 @@
         <v>18</v>
       </c>
       <c r="C184" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -2484,7 +2484,7 @@
         <v>17</v>
       </c>
       <c r="C185" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -2495,7 +2495,7 @@
         <v>17</v>
       </c>
       <c r="C186" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
@@ -2506,7 +2506,7 @@
         <v>17</v>
       </c>
       <c r="C187" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -2517,7 +2517,7 @@
         <v>16</v>
       </c>
       <c r="C188" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -2528,7 +2528,7 @@
         <v>16</v>
       </c>
       <c r="C189" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -2539,7 +2539,7 @@
         <v>15</v>
       </c>
       <c r="C190" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -2550,7 +2550,7 @@
         <v>15</v>
       </c>
       <c r="C191" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -2561,7 +2561,7 @@
         <v>15</v>
       </c>
       <c r="C192" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -2572,7 +2572,7 @@
         <v>14</v>
       </c>
       <c r="C193" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
@@ -2583,7 +2583,7 @@
         <v>14</v>
       </c>
       <c r="C194" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -2594,7 +2594,7 @@
         <v>14</v>
       </c>
       <c r="C195" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -2605,7 +2605,7 @@
         <v>13</v>
       </c>
       <c r="C196" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -2616,7 +2616,7 @@
         <v>13</v>
       </c>
       <c r="C197" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -2627,7 +2627,7 @@
         <v>13</v>
       </c>
       <c r="C198" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -2638,7 +2638,7 @@
         <v>12</v>
       </c>
       <c r="C199" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -2649,7 +2649,7 @@
         <v>12</v>
       </c>
       <c r="C200" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -2660,7 +2660,7 @@
         <v>12</v>
       </c>
       <c r="C201" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
@@ -2671,7 +2671,7 @@
         <v>11</v>
       </c>
       <c r="C202" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -2682,7 +2682,7 @@
         <v>11</v>
       </c>
       <c r="C203" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -2693,7 +2693,7 @@
         <v>11</v>
       </c>
       <c r="C204" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -2704,7 +2704,7 @@
         <v>10</v>
       </c>
       <c r="C205" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -2715,7 +2715,7 @@
         <v>10</v>
       </c>
       <c r="C206" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -2726,7 +2726,7 @@
         <v>10</v>
       </c>
       <c r="C207" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -2737,7 +2737,7 @@
         <v>9</v>
       </c>
       <c r="C208" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
@@ -2748,7 +2748,7 @@
         <v>9</v>
       </c>
       <c r="C209" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
@@ -2759,7 +2759,7 @@
         <v>9</v>
       </c>
       <c r="C210" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -2770,7 +2770,7 @@
         <v>8</v>
       </c>
       <c r="C211" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
@@ -2781,7 +2781,7 @@
         <v>8</v>
       </c>
       <c r="C212" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -2792,7 +2792,7 @@
         <v>8</v>
       </c>
       <c r="C213" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -2803,7 +2803,7 @@
         <v>7</v>
       </c>
       <c r="C214" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -2814,7 +2814,7 @@
         <v>7</v>
       </c>
       <c r="C215" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -2825,7 +2825,7 @@
         <v>7</v>
       </c>
       <c r="C216" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -2836,7 +2836,7 @@
         <v>6</v>
       </c>
       <c r="C217" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
@@ -2847,7 +2847,7 @@
         <v>6</v>
       </c>
       <c r="C218" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
@@ -2858,7 +2858,7 @@
         <v>6</v>
       </c>
       <c r="C219" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
@@ -2869,7 +2869,7 @@
         <v>5</v>
       </c>
       <c r="C220" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -2880,7 +2880,7 @@
         <v>5</v>
       </c>
       <c r="C221" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
@@ -2891,7 +2891,7 @@
         <v>5</v>
       </c>
       <c r="C222" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
@@ -2902,7 +2902,7 @@
         <v>4</v>
       </c>
       <c r="C223" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
@@ -2913,7 +2913,7 @@
         <v>4</v>
       </c>
       <c r="C224" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -2924,7 +2924,7 @@
         <v>4</v>
       </c>
       <c r="C225" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
@@ -2935,7 +2935,7 @@
         <v>3</v>
       </c>
       <c r="C226" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
@@ -2946,7 +2946,7 @@
         <v>3</v>
       </c>
       <c r="C227" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
@@ -2957,7 +2957,7 @@
         <v>3</v>
       </c>
       <c r="C228" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
@@ -2968,7 +2968,7 @@
         <v>3</v>
       </c>
       <c r="C229" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
@@ -2979,7 +2979,7 @@
         <v>3</v>
       </c>
       <c r="C230" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
@@ -2990,7 +2990,7 @@
         <v>3</v>
       </c>
       <c r="C231" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
@@ -3001,7 +3001,7 @@
         <v>3</v>
       </c>
       <c r="C232" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
@@ -3012,7 +3012,7 @@
         <v>3</v>
       </c>
       <c r="C233" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -3023,7 +3023,7 @@
         <v>3</v>
       </c>
       <c r="C234" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
@@ -3034,7 +3034,7 @@
         <v>3</v>
       </c>
       <c r="C235" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
@@ -3325,6 +3325,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3686,7 +3687,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -3694,7 +3695,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -3702,7 +3703,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -3710,7 +3711,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -3718,7 +3719,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -3726,7 +3727,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="1">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -3798,7 +3799,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -3806,7 +3807,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -3814,7 +3815,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -3822,7 +3823,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -3830,7 +3831,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -3838,7 +3839,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -3846,7 +3847,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -3854,7 +3855,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="1">
-        <v>200</v>
+        <v>215</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -3862,7 +3863,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -3870,7 +3871,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -3878,7 +3879,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -3886,7 +3887,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -3894,7 +3895,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="1">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -3902,7 +3903,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -3910,7 +3911,7 @@
         <v>70</v>
       </c>
       <c r="B72" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -3918,7 +3919,7 @@
         <v>71</v>
       </c>
       <c r="B73" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -3926,7 +3927,7 @@
         <v>72</v>
       </c>
       <c r="B74" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -3934,7 +3935,7 @@
         <v>73</v>
       </c>
       <c r="B75" s="1">
-        <v>145</v>
+        <v>125</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -3942,7 +3943,7 @@
         <v>74</v>
       </c>
       <c r="B76" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -3950,7 +3951,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -3958,7 +3959,7 @@
         <v>76</v>
       </c>
       <c r="B78" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -3966,7 +3967,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -3974,7 +3975,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -3982,7 +3983,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="1">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -3990,7 +3991,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -3998,7 +3999,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -4006,7 +4007,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -4014,7 +4015,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -4022,7 +4023,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -4030,7 +4031,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -4038,7 +4039,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -4046,7 +4047,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="1">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -4054,7 +4055,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -4062,7 +4063,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -4070,7 +4071,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -4078,7 +4079,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -4086,7 +4087,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -4094,7 +4095,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -4102,7 +4103,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -4110,7 +4111,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="1">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -4118,7 +4119,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -4126,7 +4127,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -4134,7 +4135,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -4142,7 +4143,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -4150,7 +4151,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -4158,7 +4159,7 @@
         <v>101</v>
       </c>
       <c r="B103" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -4166,7 +4167,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -4174,7 +4175,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -4182,7 +4183,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -4190,7 +4191,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
@@ -4198,7 +4199,7 @@
         <v>106</v>
       </c>
       <c r="B108" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
@@ -4206,7 +4207,7 @@
         <v>107</v>
       </c>
       <c r="B109" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -4214,7 +4215,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -4222,7 +4223,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -4230,7 +4231,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -4238,7 +4239,7 @@
         <v>111</v>
       </c>
       <c r="B113" s="1">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -4246,7 +4247,7 @@
         <v>112</v>
       </c>
       <c r="B114" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -4254,7 +4255,7 @@
         <v>113</v>
       </c>
       <c r="B115" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -4262,7 +4263,7 @@
         <v>114</v>
       </c>
       <c r="B116" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -4270,7 +4271,7 @@
         <v>115</v>
       </c>
       <c r="B117" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
@@ -4278,7 +4279,7 @@
         <v>116</v>
       </c>
       <c r="B118" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -4286,7 +4287,7 @@
         <v>117</v>
       </c>
       <c r="B119" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -4294,7 +4295,7 @@
         <v>118</v>
       </c>
       <c r="B120" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -4302,7 +4303,7 @@
         <v>119</v>
       </c>
       <c r="B121" s="1">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -4310,7 +4311,7 @@
         <v>120</v>
       </c>
       <c r="B122" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
@@ -4318,7 +4319,7 @@
         <v>121</v>
       </c>
       <c r="B123" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
@@ -4326,7 +4327,7 @@
         <v>122</v>
       </c>
       <c r="B124" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
@@ -4334,7 +4335,7 @@
         <v>123</v>
       </c>
       <c r="B125" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -4342,7 +4343,7 @@
         <v>124</v>
       </c>
       <c r="B126" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
@@ -4350,7 +4351,7 @@
         <v>125</v>
       </c>
       <c r="B127" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -4358,7 +4359,7 @@
         <v>126</v>
       </c>
       <c r="B128" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
@@ -4366,7 +4367,7 @@
         <v>127</v>
       </c>
       <c r="B129" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
@@ -4374,7 +4375,7 @@
         <v>128</v>
       </c>
       <c r="B130" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
@@ -4382,7 +4383,7 @@
         <v>129</v>
       </c>
       <c r="B131" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
@@ -4390,7 +4391,7 @@
         <v>130</v>
       </c>
       <c r="B132" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
@@ -4398,7 +4399,7 @@
         <v>131</v>
       </c>
       <c r="B133" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
@@ -4406,7 +4407,7 @@
         <v>132</v>
       </c>
       <c r="B134" s="1">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
@@ -4414,7 +4415,7 @@
         <v>133</v>
       </c>
       <c r="B135" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
@@ -4422,7 +4423,7 @@
         <v>134</v>
       </c>
       <c r="B136" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
@@ -4430,7 +4431,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -4438,7 +4439,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -4446,7 +4447,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
@@ -4454,7 +4455,7 @@
         <v>138</v>
       </c>
       <c r="B140" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -4462,7 +4463,7 @@
         <v>139</v>
       </c>
       <c r="B141" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -4470,7 +4471,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
@@ -4478,7 +4479,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
@@ -4486,7 +4487,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
@@ -4494,7 +4495,7 @@
         <v>143</v>
       </c>
       <c r="B145" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
@@ -4502,7 +4503,7 @@
         <v>144</v>
       </c>
       <c r="B146" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
@@ -4510,7 +4511,7 @@
         <v>145</v>
       </c>
       <c r="B147" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
@@ -4518,7 +4519,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -4526,7 +4527,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -4534,7 +4535,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -4542,7 +4543,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -4550,7 +4551,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -4558,7 +4559,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -4566,7 +4567,7 @@
         <v>152</v>
       </c>
       <c r="B154" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -4574,7 +4575,7 @@
         <v>153</v>
       </c>
       <c r="B155" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -4582,7 +4583,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
@@ -4590,7 +4591,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
@@ -4598,7 +4599,7 @@
         <v>156</v>
       </c>
       <c r="B158" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -4606,7 +4607,7 @@
         <v>157</v>
       </c>
       <c r="B159" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
@@ -4614,7 +4615,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -4622,7 +4623,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
@@ -4630,7 +4631,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -4638,7 +4639,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -4646,7 +4647,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -4654,7 +4655,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
@@ -4662,7 +4663,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -4670,7 +4671,7 @@
         <v>165</v>
       </c>
       <c r="B167" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
@@ -4678,7 +4679,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -4686,7 +4687,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -4694,7 +4695,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
@@ -4702,7 +4703,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -4710,7 +4711,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -4718,7 +4719,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -4726,7 +4727,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -4734,7 +4735,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -4742,7 +4743,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -4750,7 +4751,7 @@
         <v>175</v>
       </c>
       <c r="B177" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -4758,7 +4759,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
@@ -4766,7 +4767,7 @@
         <v>177</v>
       </c>
       <c r="B179" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -4774,7 +4775,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
@@ -4782,7 +4783,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
@@ -4790,7 +4791,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
@@ -4798,7 +4799,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
@@ -4806,7 +4807,7 @@
         <v>182</v>
       </c>
       <c r="B184" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
@@ -4814,7 +4815,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
@@ -4822,7 +4823,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -4830,7 +4831,7 @@
         <v>185</v>
       </c>
       <c r="B187" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
@@ -4838,7 +4839,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
@@ -4846,7 +4847,7 @@
         <v>187</v>
       </c>
       <c r="B189" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
@@ -4854,7 +4855,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
@@ -4862,7 +4863,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -4870,7 +4871,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
@@ -4878,7 +4879,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
@@ -4886,7 +4887,7 @@
         <v>192</v>
       </c>
       <c r="B194" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
@@ -4894,7 +4895,7 @@
         <v>193</v>
       </c>
       <c r="B195" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
@@ -4902,7 +4903,7 @@
         <v>194</v>
       </c>
       <c r="B196" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
@@ -4910,7 +4911,7 @@
         <v>195</v>
       </c>
       <c r="B197" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
@@ -4918,7 +4919,7 @@
         <v>196</v>
       </c>
       <c r="B198" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
@@ -4926,7 +4927,7 @@
         <v>197</v>
       </c>
       <c r="B199" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
@@ -4934,7 +4935,7 @@
         <v>198</v>
       </c>
       <c r="B200" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -4942,7 +4943,7 @@
         <v>199</v>
       </c>
       <c r="B201" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -4950,7 +4951,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
@@ -4958,7 +4959,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
@@ -4966,7 +4967,7 @@
         <v>202</v>
       </c>
       <c r="B204" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
@@ -4974,7 +4975,7 @@
         <v>203</v>
       </c>
       <c r="B205" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
@@ -4982,7 +4983,7 @@
         <v>204</v>
       </c>
       <c r="B206" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
@@ -4990,7 +4991,7 @@
         <v>205</v>
       </c>
       <c r="B207" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
@@ -4998,7 +4999,7 @@
         <v>206</v>
       </c>
       <c r="B208" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
@@ -5006,7 +5007,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
@@ -5014,7 +5015,7 @@
         <v>208</v>
       </c>
       <c r="B210" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
@@ -5022,7 +5023,7 @@
         <v>209</v>
       </c>
       <c r="B211" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
@@ -5030,7 +5031,7 @@
         <v>210</v>
       </c>
       <c r="B212" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
@@ -5038,7 +5039,7 @@
         <v>211</v>
       </c>
       <c r="B213" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
@@ -5046,7 +5047,7 @@
         <v>212</v>
       </c>
       <c r="B214" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
@@ -5054,7 +5055,7 @@
         <v>213</v>
       </c>
       <c r="B215" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
@@ -5062,7 +5063,7 @@
         <v>214</v>
       </c>
       <c r="B216" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
@@ -5070,7 +5071,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -5078,7 +5079,7 @@
         <v>216</v>
       </c>
       <c r="B218" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -5086,7 +5087,7 @@
         <v>217</v>
       </c>
       <c r="B219" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -5094,7 +5095,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -5102,7 +5103,7 @@
         <v>219</v>
       </c>
       <c r="B221" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -5110,7 +5111,7 @@
         <v>220</v>
       </c>
       <c r="B222" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -5118,7 +5119,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
@@ -5126,7 +5127,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
@@ -5134,7 +5135,7 @@
         <v>223</v>
       </c>
       <c r="B225" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
@@ -5142,7 +5143,7 @@
         <v>224</v>
       </c>
       <c r="B226" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
@@ -5150,7 +5151,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
@@ -5158,7 +5159,7 @@
         <v>226</v>
       </c>
       <c r="B228" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
@@ -5166,7 +5167,7 @@
         <v>227</v>
       </c>
       <c r="B229" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
@@ -5174,7 +5175,7 @@
         <v>228</v>
       </c>
       <c r="B230" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
@@ -5182,7 +5183,7 @@
         <v>229</v>
       </c>
       <c r="B231" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -5190,7 +5191,7 @@
         <v>230</v>
       </c>
       <c r="B232" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
@@ -5198,7 +5199,7 @@
         <v>231</v>
       </c>
       <c r="B233" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -5206,7 +5207,7 @@
         <v>232</v>
       </c>
       <c r="B234" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
@@ -5214,7 +5215,7 @@
         <v>233</v>
       </c>
       <c r="B235" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update future draft pick value, fix RB3 need ratings, update future test pick order to match current year order
</commit_message>
<xml_diff>
--- a/Files/TestFiles/DraftPickValue.xlsx
+++ b/Files/TestFiles/DraftPickValue.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="617" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF9FAFB-2AF4-4E17-A89D-BCA96B683724}"/>
+  <xr:revisionPtr revIDLastSave="844" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48427602-D899-40BC-933B-C532A7797432}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B6B8C1A-1A59-46A0-9756-E6597FCDBA38}"/>
   </bookViews>
@@ -98,13 +98,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -445,14 +448,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E893235-A107-43E5-AA8C-897A724457D3}">
-  <dimension ref="A1:C261"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="1" customWidth="1"/>
+    <col min="3" max="5" width="14.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -462,8 +465,10 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -471,10 +476,16 @@
         <v>3000</v>
       </c>
       <c r="C2" s="1">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1500</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -482,10 +493,13 @@
         <v>2600</v>
       </c>
       <c r="C3" s="1">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1400</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -493,10 +507,13 @@
         <v>2200</v>
       </c>
       <c r="C4" s="1">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1350</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -504,10 +521,13 @@
         <v>1800</v>
       </c>
       <c r="C5" s="1">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -517,8 +537,11 @@
       <c r="C6" s="1">
         <v>1250</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -526,10 +549,13 @@
         <v>1600</v>
       </c>
       <c r="C7" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1200</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -537,10 +563,13 @@
         <v>1500</v>
       </c>
       <c r="C8" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1150</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -548,10 +577,13 @@
         <v>1400</v>
       </c>
       <c r="C9" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1100</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -559,10 +591,13 @@
         <v>1350</v>
       </c>
       <c r="C10" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1050</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -572,8 +607,11 @@
       <c r="C11" s="1">
         <v>1000</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -583,8 +621,11 @@
       <c r="C12" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -594,8 +635,11 @@
       <c r="C13" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -605,8 +649,11 @@
       <c r="C14" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -616,8 +663,11 @@
       <c r="C15" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -627,8 +677,11 @@
       <c r="C16" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -638,8 +691,11 @@
       <c r="C17" s="1">
         <v>750</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -649,8 +705,11 @@
       <c r="C18" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -660,8 +719,11 @@
       <c r="C19" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -671,8 +733,11 @@
       <c r="C20" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -682,8 +747,11 @@
       <c r="C21" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -693,8 +761,11 @@
       <c r="C22" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -704,8 +775,11 @@
       <c r="C23" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -715,8 +789,11 @@
       <c r="C24" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -726,8 +803,11 @@
       <c r="C25" s="1">
         <v>600</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -735,10 +815,13 @@
         <v>720</v>
       </c>
       <c r="C26" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>550</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -746,10 +829,13 @@
         <v>700</v>
       </c>
       <c r="C27" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <v>550</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -757,10 +843,13 @@
         <v>680</v>
       </c>
       <c r="C28" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>550</v>
+      </c>
+      <c r="E28" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -768,10 +857,13 @@
         <v>660</v>
       </c>
       <c r="C29" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>550</v>
+      </c>
+      <c r="E29" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -779,10 +871,13 @@
         <v>640</v>
       </c>
       <c r="C30" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>525</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -790,10 +885,13 @@
         <v>620</v>
       </c>
       <c r="C31" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>525</v>
+      </c>
+      <c r="E31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -801,10 +899,13 @@
         <v>600</v>
       </c>
       <c r="C32" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>525</v>
+      </c>
+      <c r="E32" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -812,10 +913,13 @@
         <v>590</v>
       </c>
       <c r="C33" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>525</v>
+      </c>
+      <c r="E33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -825,8 +929,14 @@
       <c r="C34" s="1">
         <v>350</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34" s="1">
+        <v>2</v>
+      </c>
+      <c r="E34" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -836,8 +946,11 @@
       <c r="C35" s="1">
         <v>350</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E35" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -847,8 +960,11 @@
       <c r="C36" s="1">
         <v>350</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E36" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -858,8 +974,11 @@
       <c r="C37" s="1">
         <v>350</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E37" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -869,8 +988,11 @@
       <c r="C38" s="1">
         <v>350</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E38" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -880,8 +1002,11 @@
       <c r="C39" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E39" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -891,8 +1016,11 @@
       <c r="C40" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E40" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -902,8 +1030,11 @@
       <c r="C41" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E41" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -913,8 +1044,11 @@
       <c r="C42" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E42" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -924,8 +1058,11 @@
       <c r="C43" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E43" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -935,8 +1072,11 @@
       <c r="C44" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E44" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -946,8 +1086,11 @@
       <c r="C45" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E45" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -957,8 +1100,11 @@
       <c r="C46" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E46" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -968,8 +1114,11 @@
       <c r="C47" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E47" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -979,8 +1128,11 @@
       <c r="C48" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E48" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -990,8 +1142,11 @@
       <c r="C49" s="1">
         <v>275</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E49" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -1001,8 +1156,11 @@
       <c r="C50" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E50" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -1012,8 +1170,11 @@
       <c r="C51" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E51" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -1023,8 +1184,11 @@
       <c r="C52" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E52" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -1034,8 +1198,11 @@
       <c r="C53" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E53" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -1045,8 +1212,11 @@
       <c r="C54" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E54" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -1056,8 +1226,11 @@
       <c r="C55" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E55" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -1067,8 +1240,11 @@
       <c r="C56" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E56" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>55</v>
       </c>
@@ -1078,8 +1254,11 @@
       <c r="C57" s="1">
         <v>245</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E57" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>56</v>
       </c>
@@ -1089,8 +1268,11 @@
       <c r="C58" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E58" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>57</v>
       </c>
@@ -1100,8 +1282,11 @@
       <c r="C59" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E59" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>58</v>
       </c>
@@ -1111,8 +1296,11 @@
       <c r="C60" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E60" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>59</v>
       </c>
@@ -1122,8 +1310,11 @@
       <c r="C61" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E61" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>60</v>
       </c>
@@ -1133,8 +1324,11 @@
       <c r="C62" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E62" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>61</v>
       </c>
@@ -1144,8 +1338,11 @@
       <c r="C63" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E63" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>62</v>
       </c>
@@ -1155,8 +1352,11 @@
       <c r="C64" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E64" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>63</v>
       </c>
@@ -1166,8 +1366,11 @@
       <c r="C65" s="1">
         <v>215</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E65" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -1177,8 +1380,14 @@
       <c r="C66" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D66" s="1">
+        <v>3</v>
+      </c>
+      <c r="E66" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -1188,8 +1397,11 @@
       <c r="C67" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E67" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -1199,8 +1411,11 @@
       <c r="C68" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E68" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>67</v>
       </c>
@@ -1210,8 +1425,11 @@
       <c r="C69" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E69" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>68</v>
       </c>
@@ -1221,8 +1439,11 @@
       <c r="C70" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E70" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -1232,8 +1453,11 @@
       <c r="C71" s="1">
         <v>125</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E71" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -1243,8 +1467,11 @@
       <c r="C72" s="1">
         <v>125</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E72" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -1254,8 +1481,11 @@
       <c r="C73" s="1">
         <v>125</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E73" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>72</v>
       </c>
@@ -1265,8 +1495,11 @@
       <c r="C74" s="1">
         <v>125</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E74" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -1276,8 +1509,11 @@
       <c r="C75" s="1">
         <v>125</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E75" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>74</v>
       </c>
@@ -1287,8 +1523,11 @@
       <c r="C76" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E76" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -1298,8 +1537,11 @@
       <c r="C77" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E77" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>76</v>
       </c>
@@ -1309,8 +1551,11 @@
       <c r="C78" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E78" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>77</v>
       </c>
@@ -1320,8 +1565,11 @@
       <c r="C79" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E79" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>78</v>
       </c>
@@ -1331,8 +1579,11 @@
       <c r="C80" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E80" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>79</v>
       </c>
@@ -1342,8 +1593,11 @@
       <c r="C81" s="1">
         <v>105</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E81" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>80</v>
       </c>
@@ -1353,8 +1607,11 @@
       <c r="C82" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E82" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>81</v>
       </c>
@@ -1364,8 +1621,11 @@
       <c r="C83" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E83" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>82</v>
       </c>
@@ -1375,8 +1635,11 @@
       <c r="C84" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E84" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>83</v>
       </c>
@@ -1386,8 +1649,11 @@
       <c r="C85" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E85" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>84</v>
       </c>
@@ -1397,8 +1663,11 @@
       <c r="C86" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E86" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>85</v>
       </c>
@@ -1408,8 +1677,11 @@
       <c r="C87" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E87" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>86</v>
       </c>
@@ -1419,8 +1691,11 @@
       <c r="C88" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E88" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>87</v>
       </c>
@@ -1430,8 +1705,11 @@
       <c r="C89" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E89" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>88</v>
       </c>
@@ -1439,10 +1717,13 @@
         <v>145</v>
       </c>
       <c r="C90" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E90" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>89</v>
       </c>
@@ -1450,10 +1731,13 @@
         <v>140</v>
       </c>
       <c r="C91" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E91" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>90</v>
       </c>
@@ -1461,10 +1745,13 @@
         <v>136</v>
       </c>
       <c r="C92" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E92" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>91</v>
       </c>
@@ -1472,10 +1759,13 @@
         <v>132</v>
       </c>
       <c r="C93" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E93" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>92</v>
       </c>
@@ -1483,10 +1773,13 @@
         <v>128</v>
       </c>
       <c r="C94" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E94" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>93</v>
       </c>
@@ -1494,10 +1787,13 @@
         <v>124</v>
       </c>
       <c r="C95" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E95" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>94</v>
       </c>
@@ -1505,10 +1801,13 @@
         <v>120</v>
       </c>
       <c r="C96" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E96" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>95</v>
       </c>
@@ -1516,10 +1815,13 @@
         <v>116</v>
       </c>
       <c r="C97" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E97" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>96</v>
       </c>
@@ -1527,10 +1829,13 @@
         <v>112</v>
       </c>
       <c r="C98" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E98" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>97</v>
       </c>
@@ -1538,10 +1843,13 @@
         <v>108</v>
       </c>
       <c r="C99" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E99" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>98</v>
       </c>
@@ -1549,10 +1857,13 @@
         <v>104</v>
       </c>
       <c r="C100" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E100" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>99</v>
       </c>
@@ -1560,10 +1871,13 @@
         <v>100</v>
       </c>
       <c r="C101" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E101" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>100</v>
       </c>
@@ -1571,10 +1885,13 @@
         <v>96</v>
       </c>
       <c r="C102" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="E102" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>101</v>
       </c>
@@ -1582,10 +1899,13 @@
         <v>92</v>
       </c>
       <c r="C103" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E103" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>102</v>
       </c>
@@ -1593,10 +1913,16 @@
         <v>88</v>
       </c>
       <c r="C104" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="D104" s="1">
+        <v>4</v>
+      </c>
+      <c r="E104" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>103</v>
       </c>
@@ -1604,10 +1930,13 @@
         <v>86</v>
       </c>
       <c r="C105" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E105" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>104</v>
       </c>
@@ -1615,10 +1944,13 @@
         <v>84</v>
       </c>
       <c r="C106" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E106" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>105</v>
       </c>
@@ -1626,10 +1958,13 @@
         <v>82</v>
       </c>
       <c r="C107" s="1">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E107" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>106</v>
       </c>
@@ -1637,10 +1972,13 @@
         <v>80</v>
       </c>
       <c r="C108" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E108" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>107</v>
       </c>
@@ -1648,10 +1986,13 @@
         <v>78</v>
       </c>
       <c r="C109" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E109" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>108</v>
       </c>
@@ -1659,10 +2000,13 @@
         <v>76</v>
       </c>
       <c r="C110" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E110" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>109</v>
       </c>
@@ -1670,10 +2014,13 @@
         <v>74</v>
       </c>
       <c r="C111" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E111" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>110</v>
       </c>
@@ -1681,10 +2028,13 @@
         <v>72</v>
       </c>
       <c r="C112" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E112" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>111</v>
       </c>
@@ -1692,10 +2042,13 @@
         <v>70</v>
       </c>
       <c r="C113" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E113" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>112</v>
       </c>
@@ -1703,10 +2056,13 @@
         <v>68</v>
       </c>
       <c r="C114" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E114" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>113</v>
       </c>
@@ -1714,10 +2070,13 @@
         <v>66</v>
       </c>
       <c r="C115" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E115" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>114</v>
       </c>
@@ -1725,10 +2084,13 @@
         <v>64</v>
       </c>
       <c r="C116" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E116" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>115</v>
       </c>
@@ -1736,10 +2098,13 @@
         <v>62</v>
       </c>
       <c r="C117" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E117" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>116</v>
       </c>
@@ -1747,10 +2112,13 @@
         <v>60</v>
       </c>
       <c r="C118" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E118" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>117</v>
       </c>
@@ -1758,10 +2126,13 @@
         <v>58</v>
       </c>
       <c r="C119" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E119" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>118</v>
       </c>
@@ -1769,10 +2140,13 @@
         <v>56</v>
       </c>
       <c r="C120" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E120" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>119</v>
       </c>
@@ -1780,10 +2154,13 @@
         <v>54</v>
       </c>
       <c r="C121" s="1">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E121" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>120</v>
       </c>
@@ -1791,10 +2168,13 @@
         <v>52</v>
       </c>
       <c r="C122" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E122" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>121</v>
       </c>
@@ -1802,10 +2182,13 @@
         <v>50</v>
       </c>
       <c r="C123" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E123" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>122</v>
       </c>
@@ -1813,10 +2196,13 @@
         <v>49</v>
       </c>
       <c r="C124" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E124" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>123</v>
       </c>
@@ -1824,10 +2210,13 @@
         <v>48</v>
       </c>
       <c r="C125" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E125" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>124</v>
       </c>
@@ -1835,10 +2224,13 @@
         <v>47</v>
       </c>
       <c r="C126" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E126" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>125</v>
       </c>
@@ -1846,10 +2238,13 @@
         <v>46</v>
       </c>
       <c r="C127" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E127" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>126</v>
       </c>
@@ -1857,10 +2252,13 @@
         <v>45</v>
       </c>
       <c r="C128" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E128" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>127</v>
       </c>
@@ -1868,10 +2266,13 @@
         <v>44</v>
       </c>
       <c r="C129" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E129" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>128</v>
       </c>
@@ -1879,10 +2280,13 @@
         <v>43</v>
       </c>
       <c r="C130" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="E130" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>129</v>
       </c>
@@ -1890,10 +2294,13 @@
         <v>42</v>
       </c>
       <c r="C131" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="E131" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>130</v>
       </c>
@@ -1901,10 +2308,13 @@
         <v>41</v>
       </c>
       <c r="C132" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="E132" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>131</v>
       </c>
@@ -1912,10 +2322,13 @@
         <v>40</v>
       </c>
       <c r="C133" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="E133" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>132</v>
       </c>
@@ -1923,10 +2336,13 @@
         <v>39</v>
       </c>
       <c r="C134" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="E134" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>133</v>
       </c>
@@ -1934,10 +2350,13 @@
         <v>39</v>
       </c>
       <c r="C135" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E135" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>134</v>
       </c>
@@ -1945,10 +2364,13 @@
         <v>38</v>
       </c>
       <c r="C136" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E136" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>135</v>
       </c>
@@ -1956,10 +2378,13 @@
         <v>38</v>
       </c>
       <c r="C137" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E137" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>136</v>
       </c>
@@ -1967,10 +2392,13 @@
         <v>37</v>
       </c>
       <c r="C138" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E138" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>137</v>
       </c>
@@ -1978,10 +2406,13 @@
         <v>37</v>
       </c>
       <c r="C139" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E139" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>138</v>
       </c>
@@ -1989,10 +2420,13 @@
         <v>36</v>
       </c>
       <c r="C140" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="E140" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>139</v>
       </c>
@@ -2000,10 +2434,13 @@
         <v>36</v>
       </c>
       <c r="C141" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="E141" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>140</v>
       </c>
@@ -2011,10 +2448,16 @@
         <v>35</v>
       </c>
       <c r="C142" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="D142" s="1">
+        <v>5</v>
+      </c>
+      <c r="E142" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>141</v>
       </c>
@@ -2022,10 +2465,13 @@
         <v>35</v>
       </c>
       <c r="C143" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="E143" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>142</v>
       </c>
@@ -2033,10 +2479,13 @@
         <v>34</v>
       </c>
       <c r="C144" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="E144" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>143</v>
       </c>
@@ -2044,10 +2493,13 @@
         <v>34</v>
       </c>
       <c r="C145" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="E145" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>144</v>
       </c>
@@ -2055,10 +2507,13 @@
         <v>33</v>
       </c>
       <c r="C146" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E146" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>145</v>
       </c>
@@ -2066,10 +2521,13 @@
         <v>33</v>
       </c>
       <c r="C147" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E147" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>146</v>
       </c>
@@ -2077,10 +2535,13 @@
         <v>32</v>
       </c>
       <c r="C148" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E148" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>147</v>
       </c>
@@ -2088,10 +2549,13 @@
         <v>32</v>
       </c>
       <c r="C149" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E149" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>148</v>
       </c>
@@ -2099,10 +2563,13 @@
         <v>31</v>
       </c>
       <c r="C150" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E150" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>149</v>
       </c>
@@ -2110,10 +2577,13 @@
         <v>31</v>
       </c>
       <c r="C151" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E151" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>150</v>
       </c>
@@ -2121,10 +2591,13 @@
         <v>31</v>
       </c>
       <c r="C152" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E152" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>151</v>
       </c>
@@ -2132,10 +2605,13 @@
         <v>30</v>
       </c>
       <c r="C153" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="E153" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>152</v>
       </c>
@@ -2143,10 +2619,13 @@
         <v>30</v>
       </c>
       <c r="C154" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E154" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>153</v>
       </c>
@@ -2154,10 +2633,13 @@
         <v>29</v>
       </c>
       <c r="C155" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E155" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>154</v>
       </c>
@@ -2165,10 +2647,13 @@
         <v>29</v>
       </c>
       <c r="C156" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E156" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>155</v>
       </c>
@@ -2176,10 +2661,13 @@
         <v>29</v>
       </c>
       <c r="C157" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E157" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>156</v>
       </c>
@@ -2187,10 +2675,13 @@
         <v>28</v>
       </c>
       <c r="C158" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E158" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>157</v>
       </c>
@@ -2198,10 +2689,13 @@
         <v>28</v>
       </c>
       <c r="C159" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E159" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>158</v>
       </c>
@@ -2209,10 +2703,13 @@
         <v>27</v>
       </c>
       <c r="C160" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E160" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>159</v>
       </c>
@@ -2220,10 +2717,13 @@
         <v>27</v>
       </c>
       <c r="C161" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="E161" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>160</v>
       </c>
@@ -2231,10 +2731,13 @@
         <v>27</v>
       </c>
       <c r="C162" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E162" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>161</v>
       </c>
@@ -2242,10 +2745,13 @@
         <v>26</v>
       </c>
       <c r="C163" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E163" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>162</v>
       </c>
@@ -2253,10 +2759,13 @@
         <v>26</v>
       </c>
       <c r="C164" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E164" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>163</v>
       </c>
@@ -2264,10 +2773,13 @@
         <v>25</v>
       </c>
       <c r="C165" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E165" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>164</v>
       </c>
@@ -2275,10 +2787,13 @@
         <v>25</v>
       </c>
       <c r="C166" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E166" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>165</v>
       </c>
@@ -2286,10 +2801,13 @@
         <v>25</v>
       </c>
       <c r="C167" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E167" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>166</v>
       </c>
@@ -2297,10 +2815,13 @@
         <v>24</v>
       </c>
       <c r="C168" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E168" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>167</v>
       </c>
@@ -2308,10 +2829,13 @@
         <v>24</v>
       </c>
       <c r="C169" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E169" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>168</v>
       </c>
@@ -2319,10 +2843,13 @@
         <v>23</v>
       </c>
       <c r="C170" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E170" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>169</v>
       </c>
@@ -2330,10 +2857,13 @@
         <v>23</v>
       </c>
       <c r="C171" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E171" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>170</v>
       </c>
@@ -2341,10 +2871,13 @@
         <v>23</v>
       </c>
       <c r="C172" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E172" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>171</v>
       </c>
@@ -2352,10 +2885,13 @@
         <v>22</v>
       </c>
       <c r="C173" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E173" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>172</v>
       </c>
@@ -2363,10 +2899,13 @@
         <v>22</v>
       </c>
       <c r="C174" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E174" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>173</v>
       </c>
@@ -2374,10 +2913,13 @@
         <v>21</v>
       </c>
       <c r="C175" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E175" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>174</v>
       </c>
@@ -2385,10 +2927,13 @@
         <v>21</v>
       </c>
       <c r="C176" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E176" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>175</v>
       </c>
@@ -2396,10 +2941,13 @@
         <v>21</v>
       </c>
       <c r="C177" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E177" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>176</v>
       </c>
@@ -2407,10 +2955,13 @@
         <v>20</v>
       </c>
       <c r="C178" s="1">
+        <v>4</v>
+      </c>
+      <c r="E178" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>177</v>
       </c>
@@ -2418,10 +2969,16 @@
         <v>20</v>
       </c>
       <c r="C179" s="1">
+        <v>4</v>
+      </c>
+      <c r="D179" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E179" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>178</v>
       </c>
@@ -2429,10 +2986,13 @@
         <v>19</v>
       </c>
       <c r="C180" s="1">
+        <v>4</v>
+      </c>
+      <c r="E180" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>179</v>
       </c>
@@ -2440,10 +3000,13 @@
         <v>19</v>
       </c>
       <c r="C181" s="1">
+        <v>4</v>
+      </c>
+      <c r="E181" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>180</v>
       </c>
@@ -2451,10 +3014,13 @@
         <v>19</v>
       </c>
       <c r="C182" s="1">
+        <v>4</v>
+      </c>
+      <c r="E182" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
         <v>181</v>
       </c>
@@ -2462,10 +3028,13 @@
         <v>18</v>
       </c>
       <c r="C183" s="1">
+        <v>4</v>
+      </c>
+      <c r="E183" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>182</v>
       </c>
@@ -2473,10 +3042,13 @@
         <v>18</v>
       </c>
       <c r="C184" s="1">
+        <v>4</v>
+      </c>
+      <c r="E184" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>183</v>
       </c>
@@ -2484,10 +3056,13 @@
         <v>17</v>
       </c>
       <c r="C185" s="1">
+        <v>4</v>
+      </c>
+      <c r="E185" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>184</v>
       </c>
@@ -2495,10 +3070,13 @@
         <v>17</v>
       </c>
       <c r="C186" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E186" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>185</v>
       </c>
@@ -2506,10 +3084,13 @@
         <v>17</v>
       </c>
       <c r="C187" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E187" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>186</v>
       </c>
@@ -2517,10 +3098,13 @@
         <v>16</v>
       </c>
       <c r="C188" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E188" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>187</v>
       </c>
@@ -2528,10 +3112,13 @@
         <v>16</v>
       </c>
       <c r="C189" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E189" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>188</v>
       </c>
@@ -2539,10 +3126,13 @@
         <v>15</v>
       </c>
       <c r="C190" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E190" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>189</v>
       </c>
@@ -2550,10 +3140,13 @@
         <v>15</v>
       </c>
       <c r="C191" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E191" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>190</v>
       </c>
@@ -2561,10 +3154,13 @@
         <v>15</v>
       </c>
       <c r="C192" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E192" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>191</v>
       </c>
@@ -2572,10 +3168,13 @@
         <v>14</v>
       </c>
       <c r="C193" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="E193" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>192</v>
       </c>
@@ -2585,8 +3184,11 @@
       <c r="C194" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E194" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>193</v>
       </c>
@@ -2596,8 +3198,11 @@
       <c r="C195" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E195" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>194</v>
       </c>
@@ -2607,8 +3212,11 @@
       <c r="C196" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E196" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>195</v>
       </c>
@@ -2618,8 +3226,11 @@
       <c r="C197" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E197" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>196</v>
       </c>
@@ -2629,8 +3240,11 @@
       <c r="C198" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E198" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>197</v>
       </c>
@@ -2640,8 +3254,11 @@
       <c r="C199" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E199" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>198</v>
       </c>
@@ -2651,8 +3268,11 @@
       <c r="C200" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E200" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
         <v>199</v>
       </c>
@@ -2662,8 +3282,11 @@
       <c r="C201" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E201" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="1">
         <v>200</v>
       </c>
@@ -2673,8 +3296,11 @@
       <c r="C202" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E202" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
         <v>201</v>
       </c>
@@ -2684,8 +3310,11 @@
       <c r="C203" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E203" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
         <v>202</v>
       </c>
@@ -2695,8 +3324,11 @@
       <c r="C204" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E204" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
         <v>203</v>
       </c>
@@ -2706,8 +3338,11 @@
       <c r="C205" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E205" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
         <v>204</v>
       </c>
@@ -2717,8 +3352,11 @@
       <c r="C206" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E206" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="1">
         <v>205</v>
       </c>
@@ -2728,8 +3366,11 @@
       <c r="C207" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E207" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="1">
         <v>206</v>
       </c>
@@ -2739,8 +3380,11 @@
       <c r="C208" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E208" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="1">
         <v>207</v>
       </c>
@@ -2750,8 +3394,11 @@
       <c r="C209" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E209" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
         <v>208</v>
       </c>
@@ -2761,8 +3408,11 @@
       <c r="C210" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E210" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="1">
         <v>209</v>
       </c>
@@ -2772,8 +3422,11 @@
       <c r="C211" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E211" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="1">
         <v>210</v>
       </c>
@@ -2783,8 +3436,11 @@
       <c r="C212" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E212" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
         <v>211</v>
       </c>
@@ -2794,8 +3450,11 @@
       <c r="C213" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E213" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
         <v>212</v>
       </c>
@@ -2805,8 +3464,11 @@
       <c r="C214" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E214" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="1">
         <v>213</v>
       </c>
@@ -2816,8 +3478,11 @@
       <c r="C215" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E215" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="1">
         <v>214</v>
       </c>
@@ -2827,8 +3492,11 @@
       <c r="C216" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E216" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="1">
         <v>215</v>
       </c>
@@ -2838,8 +3506,14 @@
       <c r="C217" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D217" s="1">
+        <v>7</v>
+      </c>
+      <c r="E217" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="1">
         <v>216</v>
       </c>
@@ -2849,8 +3523,11 @@
       <c r="C218" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E218" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="1">
         <v>217</v>
       </c>
@@ -2860,8 +3537,11 @@
       <c r="C219" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E219" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="1">
         <v>218</v>
       </c>
@@ -2871,8 +3551,11 @@
       <c r="C220" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E220" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="1">
         <v>219</v>
       </c>
@@ -2882,8 +3565,11 @@
       <c r="C221" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E221" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="1">
         <v>220</v>
       </c>
@@ -2893,8 +3579,11 @@
       <c r="C222" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E222" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <v>221</v>
       </c>
@@ -2904,8 +3593,11 @@
       <c r="C223" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E223" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="1">
         <v>222</v>
       </c>
@@ -2915,8 +3607,11 @@
       <c r="C224" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E224" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="1">
         <v>223</v>
       </c>
@@ -2926,8 +3621,11 @@
       <c r="C225" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E225" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="1">
         <v>224</v>
       </c>
@@ -2938,7 +3636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="1">
         <v>225</v>
       </c>
@@ -2949,7 +3647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="1">
         <v>226</v>
       </c>
@@ -2960,7 +3658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="1">
         <v>227</v>
       </c>
@@ -2971,7 +3669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="1">
         <v>228</v>
       </c>
@@ -2982,7 +3680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="1">
         <v>229</v>
       </c>
@@ -2993,7 +3691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="1">
         <v>230</v>
       </c>
@@ -3004,7 +3702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="1">
         <v>231</v>
       </c>
@@ -3015,7 +3713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="1">
         <v>232</v>
       </c>
@@ -3026,7 +3724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="1">
         <v>233</v>
       </c>
@@ -3037,7 +3735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
         <v>234</v>
       </c>
@@ -3048,7 +3746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="1">
         <v>235</v>
       </c>
@@ -3059,7 +3757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="1">
         <v>236</v>
       </c>
@@ -3070,7 +3768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
         <v>237</v>
       </c>
@@ -3081,7 +3779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="1">
         <v>238</v>
       </c>
@@ -3351,7 +4049,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>1250</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3359,7 +4057,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>1250</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3367,7 +4065,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>1250</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3375,7 +4073,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1">
-        <v>1250</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3391,7 +4089,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>1000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3399,7 +4097,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1">
-        <v>1000</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3407,7 +4105,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1">
-        <v>1000</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3415,7 +4113,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1">
-        <v>1000</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3543,7 +4241,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="1">
-        <v>500</v>
+        <v>550</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3551,7 +4249,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="1">
-        <v>500</v>
+        <v>550</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3559,7 +4257,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="1">
-        <v>500</v>
+        <v>550</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -3567,7 +4265,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="1">
-        <v>500</v>
+        <v>550</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3575,7 +4273,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="1">
-        <v>500</v>
+        <v>525</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3583,7 +4281,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="1">
-        <v>500</v>
+        <v>525</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -3591,7 +4289,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="1">
-        <v>500</v>
+        <v>525</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3599,7 +4297,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="1">
-        <v>500</v>
+        <v>525</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -4055,7 +4753,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -4063,7 +4761,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -4071,7 +4769,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -4079,7 +4777,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -4087,7 +4785,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -4095,7 +4793,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -4103,7 +4801,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -4111,7 +4809,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -4119,7 +4817,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="1">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -4127,7 +4825,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="1">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -4135,7 +4833,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="1">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -4143,7 +4841,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="1">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -4151,7 +4849,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="1">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -4159,7 +4857,7 @@
         <v>101</v>
       </c>
       <c r="B103" s="1">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -4167,7 +4865,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="1">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -4175,7 +4873,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="1">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -4183,7 +4881,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="1">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -4191,7 +4889,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="1">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
@@ -4199,7 +4897,7 @@
         <v>106</v>
       </c>
       <c r="B108" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
@@ -4207,7 +4905,7 @@
         <v>107</v>
       </c>
       <c r="B109" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -4215,7 +4913,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -4223,7 +4921,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -4231,7 +4929,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -4239,7 +4937,7 @@
         <v>111</v>
       </c>
       <c r="B113" s="1">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -4247,7 +4945,7 @@
         <v>112</v>
       </c>
       <c r="B114" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -4255,7 +4953,7 @@
         <v>113</v>
       </c>
       <c r="B115" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -4263,7 +4961,7 @@
         <v>114</v>
       </c>
       <c r="B116" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -4271,7 +4969,7 @@
         <v>115</v>
       </c>
       <c r="B117" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
@@ -4279,7 +4977,7 @@
         <v>116</v>
       </c>
       <c r="B118" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -4287,7 +4985,7 @@
         <v>117</v>
       </c>
       <c r="B119" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -4295,7 +4993,7 @@
         <v>118</v>
       </c>
       <c r="B120" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -4303,7 +5001,7 @@
         <v>119</v>
       </c>
       <c r="B121" s="1">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -4311,7 +5009,7 @@
         <v>120</v>
       </c>
       <c r="B122" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
@@ -4319,7 +5017,7 @@
         <v>121</v>
       </c>
       <c r="B123" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
@@ -4327,7 +5025,7 @@
         <v>122</v>
       </c>
       <c r="B124" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
@@ -4335,7 +5033,7 @@
         <v>123</v>
       </c>
       <c r="B125" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -4343,7 +5041,7 @@
         <v>124</v>
       </c>
       <c r="B126" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
@@ -4351,7 +5049,7 @@
         <v>125</v>
       </c>
       <c r="B127" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -4359,7 +5057,7 @@
         <v>126</v>
       </c>
       <c r="B128" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
@@ -4367,7 +5065,7 @@
         <v>127</v>
       </c>
       <c r="B129" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
@@ -4375,7 +5073,7 @@
         <v>128</v>
       </c>
       <c r="B130" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
@@ -4383,7 +5081,7 @@
         <v>129</v>
       </c>
       <c r="B131" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
@@ -4391,7 +5089,7 @@
         <v>130</v>
       </c>
       <c r="B132" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
@@ -4399,7 +5097,7 @@
         <v>131</v>
       </c>
       <c r="B133" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
@@ -4407,7 +5105,7 @@
         <v>132</v>
       </c>
       <c r="B134" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
@@ -4415,7 +5113,7 @@
         <v>133</v>
       </c>
       <c r="B135" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
@@ -4423,7 +5121,7 @@
         <v>134</v>
       </c>
       <c r="B136" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
@@ -4431,7 +5129,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -4439,7 +5137,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -4447,7 +5145,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
@@ -4455,7 +5153,7 @@
         <v>138</v>
       </c>
       <c r="B140" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -4463,7 +5161,7 @@
         <v>139</v>
       </c>
       <c r="B141" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -4471,7 +5169,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
@@ -4479,7 +5177,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
@@ -4487,7 +5185,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
@@ -4495,7 +5193,7 @@
         <v>143</v>
       </c>
       <c r="B145" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
@@ -4503,7 +5201,7 @@
         <v>144</v>
       </c>
       <c r="B146" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
@@ -4511,7 +5209,7 @@
         <v>145</v>
       </c>
       <c r="B147" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
@@ -4519,7 +5217,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -4527,7 +5225,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -4535,7 +5233,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -4543,7 +5241,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -4551,7 +5249,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -4559,7 +5257,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -4567,7 +5265,7 @@
         <v>152</v>
       </c>
       <c r="B154" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -4575,7 +5273,7 @@
         <v>153</v>
       </c>
       <c r="B155" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -4583,7 +5281,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
@@ -4591,7 +5289,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
@@ -4599,7 +5297,7 @@
         <v>156</v>
       </c>
       <c r="B158" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -4607,7 +5305,7 @@
         <v>157</v>
       </c>
       <c r="B159" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
@@ -4615,7 +5313,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -4623,7 +5321,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
@@ -4631,7 +5329,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -4639,7 +5337,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -4647,7 +5345,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -4655,7 +5353,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
@@ -4663,7 +5361,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -4671,7 +5369,7 @@
         <v>165</v>
       </c>
       <c r="B167" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
@@ -4679,7 +5377,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -4687,7 +5385,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -4695,7 +5393,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
@@ -4703,7 +5401,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -4711,7 +5409,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -4719,7 +5417,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -4727,7 +5425,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -4735,7 +5433,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -4743,7 +5441,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -4751,7 +5449,7 @@
         <v>175</v>
       </c>
       <c r="B177" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -4759,7 +5457,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
@@ -4767,7 +5465,7 @@
         <v>177</v>
       </c>
       <c r="B179" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -4775,7 +5473,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
@@ -4783,7 +5481,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
@@ -4791,7 +5489,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
@@ -4799,7 +5497,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
@@ -4807,7 +5505,7 @@
         <v>182</v>
       </c>
       <c r="B184" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
@@ -4815,7 +5513,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
@@ -4823,7 +5521,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -4831,7 +5529,7 @@
         <v>185</v>
       </c>
       <c r="B187" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
@@ -4839,7 +5537,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
@@ -4847,7 +5545,7 @@
         <v>187</v>
       </c>
       <c r="B189" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
@@ -4855,7 +5553,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
@@ -4863,7 +5561,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -4871,7 +5569,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
@@ -4879,7 +5577,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Tune trade-down round modifiers and portfolio multipliers; fix decimal pick values
</commit_message>
<xml_diff>
--- a/Files/TestFiles/DraftPickValue.xlsx
+++ b/Files/TestFiles/DraftPickValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="844" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48427602-D899-40BC-933B-C532A7797432}"/>
+  <xr:revisionPtr revIDLastSave="935" documentId="8_{BAE082E4-3EDC-4A3E-8372-2028FFE0FF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43BC786C-A450-4240-9132-F0A7A3338095}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B6B8C1A-1A59-46A0-9756-E6597FCDBA38}"/>
   </bookViews>
@@ -2347,7 +2347,7 @@
         <v>133</v>
       </c>
       <c r="B135" s="1">
-        <v>39</v>
+        <v>38.5</v>
       </c>
       <c r="C135" s="1">
         <v>21</v>
@@ -2375,7 +2375,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="1">
-        <v>38</v>
+        <v>37.5</v>
       </c>
       <c r="C137" s="1">
         <v>21</v>
@@ -2403,7 +2403,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="1">
-        <v>37</v>
+        <v>36.5</v>
       </c>
       <c r="C139" s="1">
         <v>21</v>
@@ -2431,7 +2431,7 @@
         <v>139</v>
       </c>
       <c r="B141" s="1">
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="C141" s="1">
         <v>19</v>
@@ -2462,7 +2462,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="1">
-        <v>35</v>
+        <v>34.5</v>
       </c>
       <c r="C143" s="1">
         <v>19</v>
@@ -2490,7 +2490,7 @@
         <v>143</v>
       </c>
       <c r="B145" s="1">
-        <v>34</v>
+        <v>33.5</v>
       </c>
       <c r="C145" s="1">
         <v>19</v>
@@ -2518,7 +2518,7 @@
         <v>145</v>
       </c>
       <c r="B147" s="1">
-        <v>33</v>
+        <v>32.5</v>
       </c>
       <c r="C147" s="1">
         <v>16</v>
@@ -2546,7 +2546,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="1">
-        <v>32</v>
+        <v>31.7</v>
       </c>
       <c r="C149" s="1">
         <v>16</v>
@@ -2560,7 +2560,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="1">
-        <v>31</v>
+        <v>31.5</v>
       </c>
       <c r="C150" s="1">
         <v>16</v>
@@ -2574,7 +2574,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="1">
-        <v>31</v>
+        <v>31.3</v>
       </c>
       <c r="C151" s="1">
         <v>16</v>
@@ -2602,7 +2602,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="1">
-        <v>30</v>
+        <v>30.5</v>
       </c>
       <c r="C153" s="1">
         <v>16</v>
@@ -2630,7 +2630,7 @@
         <v>153</v>
       </c>
       <c r="B155" s="1">
-        <v>29</v>
+        <v>29.5</v>
       </c>
       <c r="C155" s="1">
         <v>13</v>
@@ -2658,7 +2658,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="1">
-        <v>29</v>
+        <v>28.7</v>
       </c>
       <c r="C157" s="1">
         <v>13</v>
@@ -2672,7 +2672,7 @@
         <v>156</v>
       </c>
       <c r="B158" s="1">
-        <v>28</v>
+        <v>28.3</v>
       </c>
       <c r="C158" s="1">
         <v>13</v>
@@ -2700,7 +2700,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="1">
-        <v>27</v>
+        <v>27.7</v>
       </c>
       <c r="C160" s="1">
         <v>13</v>
@@ -2714,7 +2714,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="1">
-        <v>27</v>
+        <v>27.3</v>
       </c>
       <c r="C161" s="1">
         <v>13</v>
@@ -2742,7 +2742,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="1">
-        <v>26</v>
+        <v>26.5</v>
       </c>
       <c r="C163" s="1">
         <v>9</v>
@@ -2770,7 +2770,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="1">
-        <v>25</v>
+        <v>25.7</v>
       </c>
       <c r="C165" s="1">
         <v>9</v>
@@ -2784,7 +2784,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="1">
-        <v>25</v>
+        <v>25.3</v>
       </c>
       <c r="C166" s="1">
         <v>9</v>
@@ -2812,7 +2812,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="1">
-        <v>24</v>
+        <v>24.5</v>
       </c>
       <c r="C168" s="1">
         <v>7</v>
@@ -2840,7 +2840,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="1">
-        <v>23</v>
+        <v>23.7</v>
       </c>
       <c r="C170" s="1">
         <v>7</v>
@@ -2854,7 +2854,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="1">
-        <v>23</v>
+        <v>23.3</v>
       </c>
       <c r="C171" s="1">
         <v>7</v>
@@ -2882,7 +2882,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="1">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="C173" s="1">
         <v>5</v>
@@ -2910,7 +2910,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="1">
-        <v>21</v>
+        <v>21.7</v>
       </c>
       <c r="C175" s="1">
         <v>5</v>
@@ -2924,7 +2924,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="1">
-        <v>21</v>
+        <v>21.3</v>
       </c>
       <c r="C176" s="1">
         <v>5</v>
@@ -2952,7 +2952,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="1">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="C178" s="1">
         <v>4</v>
@@ -2983,7 +2983,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="1">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="C180" s="1">
         <v>4</v>
@@ -2997,7 +2997,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="1">
-        <v>19</v>
+        <v>19.3</v>
       </c>
       <c r="C181" s="1">
         <v>4</v>
@@ -3025,7 +3025,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="1">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="C183" s="1">
         <v>4</v>
@@ -3053,7 +3053,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="1">
-        <v>17</v>
+        <v>17.7</v>
       </c>
       <c r="C185" s="1">
         <v>4</v>
@@ -3067,7 +3067,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="1">
-        <v>17</v>
+        <v>17.3</v>
       </c>
       <c r="C186" s="1">
         <v>3</v>
@@ -3095,7 +3095,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="1">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="C188" s="1">
         <v>3</v>
@@ -3123,7 +3123,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="1">
-        <v>15</v>
+        <v>15.7</v>
       </c>
       <c r="C190" s="1">
         <v>3</v>
@@ -3137,7 +3137,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="1">
-        <v>15</v>
+        <v>15.3</v>
       </c>
       <c r="C191" s="1">
         <v>3</v>
@@ -3165,7 +3165,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="1">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="C193" s="1">
         <v>3</v>
@@ -3179,7 +3179,7 @@
         <v>192</v>
       </c>
       <c r="B194" s="1">
-        <v>14</v>
+        <v>14.3</v>
       </c>
       <c r="C194" s="1">
         <v>2</v>
@@ -3207,7 +3207,7 @@
         <v>194</v>
       </c>
       <c r="B196" s="1">
-        <v>13</v>
+        <v>13.7</v>
       </c>
       <c r="C196" s="1">
         <v>2</v>
@@ -3221,7 +3221,7 @@
         <v>195</v>
       </c>
       <c r="B197" s="1">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="C197" s="1">
         <v>2</v>
@@ -3249,7 +3249,7 @@
         <v>197</v>
       </c>
       <c r="B199" s="1">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="C199" s="1">
         <v>2</v>
@@ -3263,7 +3263,7 @@
         <v>198</v>
       </c>
       <c r="B200" s="1">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="C200" s="1">
         <v>2</v>
@@ -3291,7 +3291,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="1">
-        <v>11</v>
+        <v>11.7</v>
       </c>
       <c r="C202" s="1">
         <v>2</v>
@@ -3305,7 +3305,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="1">
-        <v>11</v>
+        <v>11.3</v>
       </c>
       <c r="C203" s="1">
         <v>2</v>
@@ -3333,7 +3333,7 @@
         <v>203</v>
       </c>
       <c r="B205" s="1">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="C205" s="1">
         <v>1</v>
@@ -3347,7 +3347,7 @@
         <v>204</v>
       </c>
       <c r="B206" s="1">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="C206" s="1">
         <v>1</v>
@@ -3375,7 +3375,7 @@
         <v>206</v>
       </c>
       <c r="B208" s="1">
-        <v>9</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="C208" s="1">
         <v>1</v>
@@ -3389,7 +3389,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="1">
-        <v>9</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="C209" s="1">
         <v>1</v>
@@ -3417,7 +3417,7 @@
         <v>209</v>
       </c>
       <c r="B211" s="1">
-        <v>8</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="C211" s="1">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         <v>210</v>
       </c>
       <c r="B212" s="1">
-        <v>8</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C212" s="1">
         <v>1</v>
@@ -3459,7 +3459,7 @@
         <v>212</v>
       </c>
       <c r="B214" s="1">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="C214" s="1">
         <v>1</v>
@@ -3473,7 +3473,7 @@
         <v>213</v>
       </c>
       <c r="B215" s="1">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="C215" s="1">
         <v>1</v>
@@ -3501,7 +3501,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="1">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="C217" s="1">
         <v>1</v>
@@ -3518,7 +3518,7 @@
         <v>216</v>
       </c>
       <c r="B218" s="1">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="C218" s="1">
         <v>1</v>
@@ -3546,7 +3546,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="1">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="C220" s="1">
         <v>1</v>
@@ -3560,7 +3560,7 @@
         <v>219</v>
       </c>
       <c r="B221" s="1">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="C221" s="1">
         <v>1</v>
@@ -3588,7 +3588,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="1">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="C223" s="1">
         <v>1</v>
@@ -3602,7 +3602,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="1">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="C224" s="1">
         <v>1</v>
@@ -3630,7 +3630,7 @@
         <v>224</v>
       </c>
       <c r="B226" s="1">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="C226" s="1">
         <v>1</v>
@@ -3641,7 +3641,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="1">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="C227" s="1">
         <v>1</v>
@@ -3652,7 +3652,7 @@
         <v>226</v>
       </c>
       <c r="B228" s="1">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="C228" s="1">
         <v>1</v>
@@ -3663,7 +3663,7 @@
         <v>227</v>
       </c>
       <c r="B229" s="1">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="C229" s="1">
         <v>1</v>
@@ -3674,7 +3674,7 @@
         <v>228</v>
       </c>
       <c r="B230" s="1">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C230" s="1">
         <v>1</v>
@@ -3685,7 +3685,7 @@
         <v>229</v>
       </c>
       <c r="B231" s="1">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="C231" s="1">
         <v>1</v>
@@ -3696,7 +3696,7 @@
         <v>230</v>
       </c>
       <c r="B232" s="1">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="C232" s="1">
         <v>1</v>
@@ -3707,7 +3707,7 @@
         <v>231</v>
       </c>
       <c r="B233" s="1">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="C233" s="1">
         <v>1</v>
@@ -3718,7 +3718,7 @@
         <v>232</v>
       </c>
       <c r="B234" s="1">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="C234" s="1">
         <v>1</v>
@@ -3740,7 +3740,7 @@
         <v>234</v>
       </c>
       <c r="B236" s="1">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="C236" s="1">
         <v>1</v>
@@ -3751,7 +3751,7 @@
         <v>235</v>
       </c>
       <c r="B237" s="1">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="C237" s="1">
         <v>1</v>
@@ -3762,7 +3762,7 @@
         <v>236</v>
       </c>
       <c r="B238" s="1">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="C238" s="1">
         <v>1</v>
@@ -3773,7 +3773,7 @@
         <v>237</v>
       </c>
       <c r="B239" s="1">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="C239" s="1">
         <v>1</v>
@@ -3784,7 +3784,7 @@
         <v>238</v>
       </c>
       <c r="B240" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="C240" s="1">
         <v>1</v>
@@ -3795,7 +3795,7 @@
         <v>239</v>
       </c>
       <c r="B241" s="1">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="C241" s="1">
         <v>1</v>
@@ -3806,7 +3806,7 @@
         <v>240</v>
       </c>
       <c r="B242" s="1">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="C242" s="1">
         <v>1</v>
@@ -3817,7 +3817,7 @@
         <v>241</v>
       </c>
       <c r="B243" s="1">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="C243" s="1">
         <v>1</v>
@@ -3828,7 +3828,7 @@
         <v>242</v>
       </c>
       <c r="B244" s="1">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="C244" s="1">
         <v>1</v>
@@ -3850,7 +3850,7 @@
         <v>244</v>
       </c>
       <c r="B246" s="1">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="C246" s="1">
         <v>1</v>
@@ -3861,7 +3861,7 @@
         <v>245</v>
       </c>
       <c r="B247" s="1">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="C247" s="1">
         <v>1</v>
@@ -3872,7 +3872,7 @@
         <v>246</v>
       </c>
       <c r="B248" s="1">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="C248" s="1">
         <v>1</v>
@@ -3883,7 +3883,7 @@
         <v>247</v>
       </c>
       <c r="B249" s="1">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="C249" s="1">
         <v>1</v>
@@ -3894,7 +3894,7 @@
         <v>248</v>
       </c>
       <c r="B250" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C250" s="1">
         <v>1</v>
@@ -3905,7 +3905,7 @@
         <v>249</v>
       </c>
       <c r="B251" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C251" s="1">
         <v>1</v>
@@ -3916,7 +3916,7 @@
         <v>250</v>
       </c>
       <c r="B252" s="1">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="C252" s="1">
         <v>1</v>
@@ -3927,7 +3927,7 @@
         <v>251</v>
       </c>
       <c r="B253" s="1">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="C253" s="1">
         <v>1</v>
@@ -3938,7 +3938,7 @@
         <v>252</v>
       </c>
       <c r="B254" s="1">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="C254" s="1">
         <v>1</v>
@@ -3949,7 +3949,7 @@
         <v>253</v>
       </c>
       <c r="B255" s="1">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C255" s="1">
         <v>1</v>

</xml_diff>